<commit_message>
Release Hydro League Sync 0.1.1
</commit_message>
<xml_diff>
--- a/templates/league-participant-template.xlsx
+++ b/templates/league-participant-template.xlsx
@@ -2,13 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R2c68c2c90d6941dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联赛配置" sheetId="2" r:id="R9cbe14b6e1584ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学校信息" sheetId="3" r:id="R8a42ea270b2148d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="队伍账号映射" sheetId="4" r:id="Rcfaf975f004548b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题目映射" sheetId="5" r:id="R7a0fb11aae614b67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="校验汇总" sheetId="6" r:id="R6281523851354592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项字典" sheetId="7" r:id="Rac085e8a71c44f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R3aa8381845f644ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="联赛配置" sheetId="2" r:id="R60ef5815b2664e4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学校信息" sheetId="3" r:id="R9557b4d8fd02492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="队伍账号映射" sheetId="4" r:id="R199c4fcf87e4433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题目映射" sheetId="5" r:id="R6db7c31bb8864fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="校验汇总" sheetId="6" r:id="R63515a738d4048e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选项字典" sheetId="7" r:id="R3c67ad6bd3644296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="奖牌设置" sheetId="8" r:id="R77d6c104b5354bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工奖项" sheetId="9" r:id="R934543ebc2594e03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +26,7 @@
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -67,8 +69,42 @@
       <x:color rgb="FFD97706"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263746"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF285E6B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFC56A00"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF263746"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -105,8 +141,38 @@
         <x:fgColor rgb="FFF3F4F6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F2B3A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC9EBF5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0E5563"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F2F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4DE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="18">
+  <x:borders count="19">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -250,11 +316,25 @@
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD6DEE3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD6DEE3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD6DEE3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD6DEE3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -449,6 +529,60 @@
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -460,7 +594,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -471,7 +605,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -482,7 +616,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -493,7 +627,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -504,7 +638,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -515,7 +649,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -526,7 +660,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -537,7 +671,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -548,7 +682,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -559,7 +693,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -570,7 +704,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -581,7 +715,7 @@
         <x:color rgb="FFD97706"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -592,7 +726,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -603,7 +737,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -614,7 +748,7 @@
         <x:color rgb="FFD97706"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -1180,6 +1314,100 @@
       <x:c r="E17" s="34"/>
       <x:c r="F17" s="48"/>
     </x:row>
+    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="A19" s="106" t="str">
+        <x:v>可选扩展（不填写仍兼容旧四表模板）</x:v>
+      </x:c>
+      <x:c r="B19" s="106"/>
+      <x:c r="C19" s="106"/>
+      <x:c r="D19" s="106"/>
+      <x:c r="E19" s="106"/>
+      <x:c r="F19" s="106"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="109" t="str">
+        <x:v>校徽URL</x:v>
+      </x:c>
+      <x:c r="B20" s="108" t="str">
+        <x:v>“学校信息”P列填写无账号密码的完整 HTTP(S) 地址，或 /hydro-league-xcpcio/ 下的同源根相对路径；断外网机房优先使用根相对路径。</x:v>
+      </x:c>
+      <x:c r="C20" s="108"/>
+      <x:c r="D20" s="108"/>
+      <x:c r="E20" s="108"/>
+      <x:c r="F20" s="108"/>
+    </x:row>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="109" t="str">
+        <x:v>奖牌分组</x:v>
+      </x:c>
+      <x:c r="B21" s="108" t="str">
+        <x:v>“队伍账号映射”U列填写中文或英文分组，多项用半角或全角逗号分隔。</x:v>
+      </x:c>
+      <x:c r="C21" s="108"/>
+      <x:c r="D21" s="108"/>
+      <x:c r="E21" s="108"/>
+      <x:c r="F21" s="108"/>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="109" t="str">
+        <x:v>奖牌设置</x:v>
+      </x:c>
+      <x:c r="B22" s="108" t="str">
+        <x:v>可选工作表。每个分组填写金、银、铜牌显示数量；分组必须至少被一支启用队伍使用。</x:v>
+      </x:c>
+      <x:c r="C22" s="108"/>
+      <x:c r="D22" s="108"/>
+      <x:c r="E22" s="108"/>
+      <x:c r="F22" s="108"/>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="109" t="str">
+        <x:v>人工奖项</x:v>
+      </x:c>
+      <x:c r="B23" s="108" t="str">
+        <x:v>可选工作表。奖项 ID 唯一，队伍 ID 列表用逗号分隔；这里的数据原样导出到 Contest API/CDP。</x:v>
+      </x:c>
+      <x:c r="C23" s="108"/>
+      <x:c r="D23" s="108"/>
+      <x:c r="E23" s="108"/>
+      <x:c r="F23" s="108"/>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="109" t="str">
+        <x:v>停用队伍</x:v>
+      </x:c>
+      <x:c r="B24" s="108" t="str">
+        <x:v>停用队伍不会进入中心配置，也不能出现在人工奖项中；已有 Hydro 历史数据不会因此被删除。</x:v>
+      </x:c>
+      <x:c r="C24" s="108"/>
+      <x:c r="D24" s="108"/>
+      <x:c r="E24" s="108"/>
+      <x:c r="F24" s="108"/>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="109" t="str">
+        <x:v>权威关系</x:v>
+      </x:c>
+      <x:c r="B25" s="108" t="str">
+        <x:v>人工奖项名单是 Resolver 的权威数据；奖牌设置只控制 XCPCIO 的分组奖牌显示数量。</x:v>
+      </x:c>
+      <x:c r="C25" s="108"/>
+      <x:c r="D25" s="108"/>
+      <x:c r="E25" s="108"/>
+      <x:c r="F25" s="108"/>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="109" t="str">
+        <x:v>保留分组</x:v>
+      </x:c>
+      <x:c r="B26" s="108" t="str">
+        <x:v>不要手工填写 official 或 unofficial；中心服务会根据队伍类型自动生成。</x:v>
+      </x:c>
+      <x:c r="C26" s="108"/>
+      <x:c r="D26" s="108"/>
+      <x:c r="E26" s="108"/>
+      <x:c r="F26" s="108"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -1191,6 +1419,14 @@
     <x:mergeCell ref="B15:F15"/>
     <x:mergeCell ref="B16:F16"/>
     <x:mergeCell ref="B17:F17"/>
+    <x:mergeCell ref="A19:F19"/>
+    <x:mergeCell ref="B20:F20"/>
+    <x:mergeCell ref="B21:F21"/>
+    <x:mergeCell ref="B22:F22"/>
+    <x:mergeCell ref="B23:F23"/>
+    <x:mergeCell ref="B24:F24"/>
+    <x:mergeCell ref="B25:F25"/>
+    <x:mergeCell ref="B26:F26"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1410,7 +1646,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0317cffe4b81496b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe237ebc6ccb4ff7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1434,6 +1670,7 @@
     <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -1482,6 +1719,9 @@
       <x:c r="O1" s="4" t="str">
         <x:v>学校信息</x:v>
       </x:c>
+      <x:c r="P1" t="str">
+        <x:v>学校信息</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -1529,6 +1769,9 @@
       <x:c r="O2" s="8" t="str">
         <x:v>每所学校填写一行。学校ID用于Excel关联；站点ID用于同步协议，两者都必须全局唯一且建议使用小写英文。</x:v>
       </x:c>
+      <x:c r="P2" t="str">
+        <x:v>每所学校填写一行。学校ID用于Excel关联；站点ID用于同步协议，两者都必须全局唯一且建议使用小写英文。</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="20" t="str">
@@ -1575,6 +1818,9 @@
       </x:c>
       <x:c r="O3" s="22" t="str">
         <x:v>校验结果</x:v>
+      </x:c>
+      <x:c r="P3" s="87" t="str">
+        <x:v>校徽URL</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
@@ -1595,6 +1841,7 @@
       <x:c r="O4" s="59" t="str">
         <x:f>IF(COUNTA(A4:N4)=0,"",IF(OR(A4="",B4="",C4="",D4="",E4="",F4="",G4="",H4="",I4="",J4="",L4=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A4)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D4)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P4" s="91"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="63"/>
@@ -1614,6 +1861,7 @@
       <x:c r="O5" s="60" t="str">
         <x:f>IF(COUNTA(A5:N5)=0,"",IF(OR(A5="",B5="",C5="",D5="",E5="",F5="",G5="",H5="",I5="",J5="",L5=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A5)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D5)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P5" s="91"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="63"/>
@@ -1633,6 +1881,7 @@
       <x:c r="O6" s="60" t="str">
         <x:f>IF(COUNTA(A6:N6)=0,"",IF(OR(A6="",B6="",C6="",D6="",E6="",F6="",G6="",H6="",I6="",J6="",L6=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A6)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D6)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P6" s="91"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="63"/>
@@ -1652,6 +1901,7 @@
       <x:c r="O7" s="60" t="str">
         <x:f>IF(COUNTA(A7:N7)=0,"",IF(OR(A7="",B7="",C7="",D7="",E7="",F7="",G7="",H7="",I7="",J7="",L7=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A7)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D7)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P7" s="91"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="63"/>
@@ -1671,6 +1921,7 @@
       <x:c r="O8" s="60" t="str">
         <x:f>IF(COUNTA(A8:N8)=0,"",IF(OR(A8="",B8="",C8="",D8="",E8="",F8="",G8="",H8="",I8="",J8="",L8=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A8)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D8)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P8" s="91"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="63"/>
@@ -1690,6 +1941,7 @@
       <x:c r="O9" s="60" t="str">
         <x:f>IF(COUNTA(A9:N9)=0,"",IF(OR(A9="",B9="",C9="",D9="",E9="",F9="",G9="",H9="",I9="",J9="",L9=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A9)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D9)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P9" s="91"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="63"/>
@@ -1709,6 +1961,7 @@
       <x:c r="O10" s="60" t="str">
         <x:f>IF(COUNTA(A10:N10)=0,"",IF(OR(A10="",B10="",C10="",D10="",E10="",F10="",G10="",H10="",I10="",J10="",L10=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A10)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D10)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P10" s="91"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="63"/>
@@ -1728,6 +1981,7 @@
       <x:c r="O11" s="60" t="str">
         <x:f>IF(COUNTA(A11:N11)=0,"",IF(OR(A11="",B11="",C11="",D11="",E11="",F11="",G11="",H11="",I11="",J11="",L11=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A11)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D11)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P11" s="91"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="63"/>
@@ -1747,6 +2001,7 @@
       <x:c r="O12" s="60" t="str">
         <x:f>IF(COUNTA(A12:N12)=0,"",IF(OR(A12="",B12="",C12="",D12="",E12="",F12="",G12="",H12="",I12="",J12="",L12=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A12)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D12)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P12" s="91"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="63"/>
@@ -1766,6 +2021,7 @@
       <x:c r="O13" s="60" t="str">
         <x:f>IF(COUNTA(A13:N13)=0,"",IF(OR(A13="",B13="",C13="",D13="",E13="",F13="",G13="",H13="",I13="",J13="",L13=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A13)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D13)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P13" s="91"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="63"/>
@@ -1785,6 +2041,7 @@
       <x:c r="O14" s="60" t="str">
         <x:f>IF(COUNTA(A14:N14)=0,"",IF(OR(A14="",B14="",C14="",D14="",E14="",F14="",G14="",H14="",I14="",J14="",L14=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A14)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D14)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P14" s="91"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="63"/>
@@ -1804,6 +2061,7 @@
       <x:c r="O15" s="60" t="str">
         <x:f>IF(COUNTA(A15:N15)=0,"",IF(OR(A15="",B15="",C15="",D15="",E15="",F15="",G15="",H15="",I15="",J15="",L15=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A15)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D15)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P15" s="91"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="63"/>
@@ -1823,6 +2081,7 @@
       <x:c r="O16" s="60" t="str">
         <x:f>IF(COUNTA(A16:N16)=0,"",IF(OR(A16="",B16="",C16="",D16="",E16="",F16="",G16="",H16="",I16="",J16="",L16=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A16)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D16)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P16" s="91"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="63"/>
@@ -1842,6 +2101,7 @@
       <x:c r="O17" s="60" t="str">
         <x:f>IF(COUNTA(A17:N17)=0,"",IF(OR(A17="",B17="",C17="",D17="",E17="",F17="",G17="",H17="",I17="",J17="",L17=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A17)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D17)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P17" s="91"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="63"/>
@@ -1861,6 +2121,7 @@
       <x:c r="O18" s="60" t="str">
         <x:f>IF(COUNTA(A18:N18)=0,"",IF(OR(A18="",B18="",C18="",D18="",E18="",F18="",G18="",H18="",I18="",J18="",L18=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A18)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D18)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P18" s="91"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="63"/>
@@ -1880,6 +2141,7 @@
       <x:c r="O19" s="60" t="str">
         <x:f>IF(COUNTA(A19:N19)=0,"",IF(OR(A19="",B19="",C19="",D19="",E19="",F19="",G19="",H19="",I19="",J19="",L19=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A19)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D19)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P19" s="91"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="63"/>
@@ -1899,6 +2161,7 @@
       <x:c r="O20" s="60" t="str">
         <x:f>IF(COUNTA(A20:N20)=0,"",IF(OR(A20="",B20="",C20="",D20="",E20="",F20="",G20="",H20="",I20="",J20="",L20=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A20)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D20)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P20" s="91"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="63"/>
@@ -1918,6 +2181,7 @@
       <x:c r="O21" s="60" t="str">
         <x:f>IF(COUNTA(A21:N21)=0,"",IF(OR(A21="",B21="",C21="",D21="",E21="",F21="",G21="",H21="",I21="",J21="",L21=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A21)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D21)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P21" s="91"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="63"/>
@@ -1937,6 +2201,7 @@
       <x:c r="O22" s="60" t="str">
         <x:f>IF(COUNTA(A22:N22)=0,"",IF(OR(A22="",B22="",C22="",D22="",E22="",F22="",G22="",H22="",I22="",J22="",L22=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A22)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D22)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P22" s="91"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="63"/>
@@ -1956,6 +2221,7 @@
       <x:c r="O23" s="60" t="str">
         <x:f>IF(COUNTA(A23:N23)=0,"",IF(OR(A23="",B23="",C23="",D23="",E23="",F23="",G23="",H23="",I23="",J23="",L23=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A23)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D23)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P23" s="91"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="63"/>
@@ -1975,6 +2241,7 @@
       <x:c r="O24" s="60" t="str">
         <x:f>IF(COUNTA(A24:N24)=0,"",IF(OR(A24="",B24="",C24="",D24="",E24="",F24="",G24="",H24="",I24="",J24="",L24=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A24)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D24)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P24" s="91"/>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="63"/>
@@ -1994,6 +2261,7 @@
       <x:c r="O25" s="60" t="str">
         <x:f>IF(COUNTA(A25:N25)=0,"",IF(OR(A25="",B25="",C25="",D25="",E25="",F25="",G25="",H25="",I25="",J25="",L25=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A25)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D25)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P25" s="91"/>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="63"/>
@@ -2013,6 +2281,7 @@
       <x:c r="O26" s="60" t="str">
         <x:f>IF(COUNTA(A26:N26)=0,"",IF(OR(A26="",B26="",C26="",D26="",E26="",F26="",G26="",H26="",I26="",J26="",L26=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A26)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D26)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P26" s="91"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="63"/>
@@ -2032,6 +2301,7 @@
       <x:c r="O27" s="60" t="str">
         <x:f>IF(COUNTA(A27:N27)=0,"",IF(OR(A27="",B27="",C27="",D27="",E27="",F27="",G27="",H27="",I27="",J27="",L27=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A27)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D27)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P27" s="91"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="63"/>
@@ -2051,6 +2321,7 @@
       <x:c r="O28" s="60" t="str">
         <x:f>IF(COUNTA(A28:N28)=0,"",IF(OR(A28="",B28="",C28="",D28="",E28="",F28="",G28="",H28="",I28="",J28="",L28=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A28)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D28)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P28" s="91"/>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="63"/>
@@ -2070,6 +2341,7 @@
       <x:c r="O29" s="60" t="str">
         <x:f>IF(COUNTA(A29:N29)=0,"",IF(OR(A29="",B29="",C29="",D29="",E29="",F29="",G29="",H29="",I29="",J29="",L29=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A29)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D29)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P29" s="91"/>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="63"/>
@@ -2089,6 +2361,7 @@
       <x:c r="O30" s="60" t="str">
         <x:f>IF(COUNTA(A30:N30)=0,"",IF(OR(A30="",B30="",C30="",D30="",E30="",F30="",G30="",H30="",I30="",J30="",L30=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A30)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D30)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P30" s="91"/>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="63"/>
@@ -2108,6 +2381,7 @@
       <x:c r="O31" s="60" t="str">
         <x:f>IF(COUNTA(A31:N31)=0,"",IF(OR(A31="",B31="",C31="",D31="",E31="",F31="",G31="",H31="",I31="",J31="",L31=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A31)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D31)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P31" s="91"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="63"/>
@@ -2127,6 +2401,7 @@
       <x:c r="O32" s="60" t="str">
         <x:f>IF(COUNTA(A32:N32)=0,"",IF(OR(A32="",B32="",C32="",D32="",E32="",F32="",G32="",H32="",I32="",J32="",L32=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A32)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D32)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P32" s="91"/>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="63"/>
@@ -2146,6 +2421,7 @@
       <x:c r="O33" s="60" t="str">
         <x:f>IF(COUNTA(A33:N33)=0,"",IF(OR(A33="",B33="",C33="",D33="",E33="",F33="",G33="",H33="",I33="",J33="",L33=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A33)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D33)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P33" s="91"/>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="63"/>
@@ -2165,6 +2441,7 @@
       <x:c r="O34" s="60" t="str">
         <x:f>IF(COUNTA(A34:N34)=0,"",IF(OR(A34="",B34="",C34="",D34="",E34="",F34="",G34="",H34="",I34="",J34="",L34=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A34)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D34)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P34" s="91"/>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="63"/>
@@ -2184,6 +2461,7 @@
       <x:c r="O35" s="60" t="str">
         <x:f>IF(COUNTA(A35:N35)=0,"",IF(OR(A35="",B35="",C35="",D35="",E35="",F35="",G35="",H35="",I35="",J35="",L35=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A35)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D35)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P35" s="91"/>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="63"/>
@@ -2203,6 +2481,7 @@
       <x:c r="O36" s="60" t="str">
         <x:f>IF(COUNTA(A36:N36)=0,"",IF(OR(A36="",B36="",C36="",D36="",E36="",F36="",G36="",H36="",I36="",J36="",L36=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A36)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D36)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P36" s="91"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="63"/>
@@ -2222,6 +2501,7 @@
       <x:c r="O37" s="60" t="str">
         <x:f>IF(COUNTA(A37:N37)=0,"",IF(OR(A37="",B37="",C37="",D37="",E37="",F37="",G37="",H37="",I37="",J37="",L37=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A37)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D37)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P37" s="91"/>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="63"/>
@@ -2241,6 +2521,7 @@
       <x:c r="O38" s="60" t="str">
         <x:f>IF(COUNTA(A38:N38)=0,"",IF(OR(A38="",B38="",C38="",D38="",E38="",F38="",G38="",H38="",I38="",J38="",L38=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A38)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D38)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P38" s="91"/>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="63"/>
@@ -2260,6 +2541,7 @@
       <x:c r="O39" s="60" t="str">
         <x:f>IF(COUNTA(A39:N39)=0,"",IF(OR(A39="",B39="",C39="",D39="",E39="",F39="",G39="",H39="",I39="",J39="",L39=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A39)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D39)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P39" s="91"/>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="63"/>
@@ -2279,6 +2561,7 @@
       <x:c r="O40" s="60" t="str">
         <x:f>IF(COUNTA(A40:N40)=0,"",IF(OR(A40="",B40="",C40="",D40="",E40="",F40="",G40="",H40="",I40="",J40="",L40=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A40)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D40)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P40" s="91"/>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="63"/>
@@ -2298,6 +2581,7 @@
       <x:c r="O41" s="60" t="str">
         <x:f>IF(COUNTA(A41:N41)=0,"",IF(OR(A41="",B41="",C41="",D41="",E41="",F41="",G41="",H41="",I41="",J41="",L41=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A41)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D41)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P41" s="91"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="63"/>
@@ -2317,6 +2601,7 @@
       <x:c r="O42" s="60" t="str">
         <x:f>IF(COUNTA(A42:N42)=0,"",IF(OR(A42="",B42="",C42="",D42="",E42="",F42="",G42="",H42="",I42="",J42="",L42=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A42)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D42)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P42" s="91"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="63"/>
@@ -2336,6 +2621,7 @@
       <x:c r="O43" s="60" t="str">
         <x:f>IF(COUNTA(A43:N43)=0,"",IF(OR(A43="",B43="",C43="",D43="",E43="",F43="",G43="",H43="",I43="",J43="",L43=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A43)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D43)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P43" s="91"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="63"/>
@@ -2355,6 +2641,7 @@
       <x:c r="O44" s="60" t="str">
         <x:f>IF(COUNTA(A44:N44)=0,"",IF(OR(A44="",B44="",C44="",D44="",E44="",F44="",G44="",H44="",I44="",J44="",L44=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A44)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D44)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P44" s="91"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="63"/>
@@ -2374,6 +2661,7 @@
       <x:c r="O45" s="60" t="str">
         <x:f>IF(COUNTA(A45:N45)=0,"",IF(OR(A45="",B45="",C45="",D45="",E45="",F45="",G45="",H45="",I45="",J45="",L45=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A45)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D45)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P45" s="91"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="63"/>
@@ -2393,6 +2681,7 @@
       <x:c r="O46" s="60" t="str">
         <x:f>IF(COUNTA(A46:N46)=0,"",IF(OR(A46="",B46="",C46="",D46="",E46="",F46="",G46="",H46="",I46="",J46="",L46=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A46)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D46)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P46" s="91"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="63"/>
@@ -2412,6 +2701,7 @@
       <x:c r="O47" s="60" t="str">
         <x:f>IF(COUNTA(A47:N47)=0,"",IF(OR(A47="",B47="",C47="",D47="",E47="",F47="",G47="",H47="",I47="",J47="",L47=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A47)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D47)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P47" s="91"/>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="63"/>
@@ -2431,6 +2721,7 @@
       <x:c r="O48" s="60" t="str">
         <x:f>IF(COUNTA(A48:N48)=0,"",IF(OR(A48="",B48="",C48="",D48="",E48="",F48="",G48="",H48="",I48="",J48="",L48=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A48)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D48)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P48" s="91"/>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="63"/>
@@ -2450,6 +2741,7 @@
       <x:c r="O49" s="60" t="str">
         <x:f>IF(COUNTA(A49:N49)=0,"",IF(OR(A49="",B49="",C49="",D49="",E49="",F49="",G49="",H49="",I49="",J49="",L49=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A49)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D49)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P49" s="91"/>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="63"/>
@@ -2469,6 +2761,7 @@
       <x:c r="O50" s="60" t="str">
         <x:f>IF(COUNTA(A50:N50)=0,"",IF(OR(A50="",B50="",C50="",D50="",E50="",F50="",G50="",H50="",I50="",J50="",L50=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A50)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D50)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P50" s="91"/>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="63"/>
@@ -2488,6 +2781,7 @@
       <x:c r="O51" s="60" t="str">
         <x:f>IF(COUNTA(A51:N51)=0,"",IF(OR(A51="",B51="",C51="",D51="",E51="",F51="",G51="",H51="",I51="",J51="",L51=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A51)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D51)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P51" s="91"/>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="63"/>
@@ -2507,6 +2801,7 @@
       <x:c r="O52" s="60" t="str">
         <x:f>IF(COUNTA(A52:N52)=0,"",IF(OR(A52="",B52="",C52="",D52="",E52="",F52="",G52="",H52="",I52="",J52="",L52=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A52)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D52)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P52" s="91"/>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="64"/>
@@ -2526,11 +2821,12 @@
       <x:c r="O53" s="61" t="str">
         <x:f>IF(COUNTA(A53:N53)=0,"",IF(OR(A53="",B53="",C53="",D53="",E53="",F53="",G53="",H53="",I53="",J53="",L53=""),"缺少必填项",IF(COUNTIF($A$4:$A$53,A53)&gt;1,"学校ID重复",IF(COUNTIF($D$4:$D$53,D53)&gt;1,"站点ID重复","通过"))))</x:f>
       </x:c>
+      <x:c r="P53" s="91"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O1"/>
-    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="A1:P1"/>
+    <x:mergeCell ref="A2:P2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A53">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -2557,7 +2853,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e5dcc2b1e5449dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf76617a930d4141"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2586,6 +2882,7 @@
     <x:col min="18" max="18" width="14" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="26" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="21" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -2649,6 +2946,9 @@
       <x:c r="T1" s="4" t="str">
         <x:v>全局队伍 ID 与各校 Hydro 账号映射</x:v>
       </x:c>
+      <x:c r="U1" t="str">
+        <x:v>全局队伍 ID 与各校 Hydro 账号映射</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -2711,6 +3011,9 @@
       <x:c r="T2" s="8" t="str">
         <x:v>每支队伍一行。灰色的域ID和比赛ID由学校ID自动带出，请勿覆盖；同一学校的Hydro UID只能映射到一个启用队伍。</x:v>
       </x:c>
+      <x:c r="U2" t="str">
+        <x:v>每支队伍一行。灰色的域ID和比赛ID由学校ID自动带出，请勿覆盖；同一学校的Hydro UID只能映射到一个启用队伍。</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="20" t="str">
@@ -2772,6 +3075,9 @@
       </x:c>
       <x:c r="T3" s="22" t="str">
         <x:v>校验结果</x:v>
+      </x:c>
+      <x:c r="U3" s="87" t="str">
+        <x:v>奖牌分组</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
@@ -2801,6 +3107,7 @@
       <x:c r="T4" s="59" t="str">
         <x:f>IF(COUNTA(A4:D4)+COUNTA(G4:S4)=0,"",IF(OR(A4="",B4="",C4="",D4="",G4="",H4="",J4="",R4=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A4)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B4)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B4,$G$4:$G$203,G4,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U4" s="92"/>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="70"/>
@@ -2829,6 +3136,7 @@
       <x:c r="T5" s="60" t="str">
         <x:f>IF(COUNTA(A5:D5)+COUNTA(G5:S5)=0,"",IF(OR(A5="",B5="",C5="",D5="",G5="",H5="",J5="",R5=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A5)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B5)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B5,$G$4:$G$203,G5,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U5" s="91"/>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="70"/>
@@ -2857,6 +3165,7 @@
       <x:c r="T6" s="60" t="str">
         <x:f>IF(COUNTA(A6:D6)+COUNTA(G6:S6)=0,"",IF(OR(A6="",B6="",C6="",D6="",G6="",H6="",J6="",R6=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A6)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B6)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B6,$G$4:$G$203,G6,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U6" s="92"/>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="A7" s="70"/>
@@ -2885,6 +3194,7 @@
       <x:c r="T7" s="60" t="str">
         <x:f>IF(COUNTA(A7:D7)+COUNTA(G7:S7)=0,"",IF(OR(A7="",B7="",C7="",D7="",G7="",H7="",J7="",R7=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A7)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B7)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B7,$G$4:$G$203,G7,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U7" s="91"/>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
       <x:c r="A8" s="70"/>
@@ -2913,6 +3223,7 @@
       <x:c r="T8" s="60" t="str">
         <x:f>IF(COUNTA(A8:D8)+COUNTA(G8:S8)=0,"",IF(OR(A8="",B8="",C8="",D8="",G8="",H8="",J8="",R8=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A8)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B8)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B8,$G$4:$G$203,G8,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U8" s="92"/>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="70"/>
@@ -2941,6 +3252,7 @@
       <x:c r="T9" s="60" t="str">
         <x:f>IF(COUNTA(A9:D9)+COUNTA(G9:S9)=0,"",IF(OR(A9="",B9="",C9="",D9="",G9="",H9="",J9="",R9=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A9)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B9)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B9,$G$4:$G$203,G9,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U9" s="91"/>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="70"/>
@@ -2969,6 +3281,7 @@
       <x:c r="T10" s="60" t="str">
         <x:f>IF(COUNTA(A10:D10)+COUNTA(G10:S10)=0,"",IF(OR(A10="",B10="",C10="",D10="",G10="",H10="",J10="",R10=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A10)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B10)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B10,$G$4:$G$203,G10,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U10" s="92"/>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="70"/>
@@ -2997,6 +3310,7 @@
       <x:c r="T11" s="60" t="str">
         <x:f>IF(COUNTA(A11:D11)+COUNTA(G11:S11)=0,"",IF(OR(A11="",B11="",C11="",D11="",G11="",H11="",J11="",R11=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A11)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B11)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B11,$G$4:$G$203,G11,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U11" s="91"/>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="70"/>
@@ -3025,6 +3339,7 @@
       <x:c r="T12" s="60" t="str">
         <x:f>IF(COUNTA(A12:D12)+COUNTA(G12:S12)=0,"",IF(OR(A12="",B12="",C12="",D12="",G12="",H12="",J12="",R12=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A12)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B12)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B12,$G$4:$G$203,G12,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U12" s="92"/>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="70"/>
@@ -3053,6 +3368,7 @@
       <x:c r="T13" s="60" t="str">
         <x:f>IF(COUNTA(A13:D13)+COUNTA(G13:S13)=0,"",IF(OR(A13="",B13="",C13="",D13="",G13="",H13="",J13="",R13=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A13)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B13)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B13,$G$4:$G$203,G13,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U13" s="91"/>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="70"/>
@@ -3081,6 +3397,7 @@
       <x:c r="T14" s="60" t="str">
         <x:f>IF(COUNTA(A14:D14)+COUNTA(G14:S14)=0,"",IF(OR(A14="",B14="",C14="",D14="",G14="",H14="",J14="",R14=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A14)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B14)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B14,$G$4:$G$203,G14,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U14" s="92"/>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="70"/>
@@ -3109,6 +3426,7 @@
       <x:c r="T15" s="60" t="str">
         <x:f>IF(COUNTA(A15:D15)+COUNTA(G15:S15)=0,"",IF(OR(A15="",B15="",C15="",D15="",G15="",H15="",J15="",R15=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A15)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B15)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B15,$G$4:$G$203,G15,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U15" s="91"/>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="70"/>
@@ -3137,6 +3455,7 @@
       <x:c r="T16" s="60" t="str">
         <x:f>IF(COUNTA(A16:D16)+COUNTA(G16:S16)=0,"",IF(OR(A16="",B16="",C16="",D16="",G16="",H16="",J16="",R16=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A16)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B16)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B16,$G$4:$G$203,G16,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U16" s="92"/>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="70"/>
@@ -3165,6 +3484,7 @@
       <x:c r="T17" s="60" t="str">
         <x:f>IF(COUNTA(A17:D17)+COUNTA(G17:S17)=0,"",IF(OR(A17="",B17="",C17="",D17="",G17="",H17="",J17="",R17=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A17)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B17)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B17,$G$4:$G$203,G17,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U17" s="91"/>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="70"/>
@@ -3193,6 +3513,7 @@
       <x:c r="T18" s="60" t="str">
         <x:f>IF(COUNTA(A18:D18)+COUNTA(G18:S18)=0,"",IF(OR(A18="",B18="",C18="",D18="",G18="",H18="",J18="",R18=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A18)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B18)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B18,$G$4:$G$203,G18,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U18" s="92"/>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="70"/>
@@ -3221,6 +3542,7 @@
       <x:c r="T19" s="60" t="str">
         <x:f>IF(COUNTA(A19:D19)+COUNTA(G19:S19)=0,"",IF(OR(A19="",B19="",C19="",D19="",G19="",H19="",J19="",R19=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A19)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B19)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B19,$G$4:$G$203,G19,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U19" s="91"/>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="70"/>
@@ -3249,6 +3571,7 @@
       <x:c r="T20" s="60" t="str">
         <x:f>IF(COUNTA(A20:D20)+COUNTA(G20:S20)=0,"",IF(OR(A20="",B20="",C20="",D20="",G20="",H20="",J20="",R20=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A20)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B20)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B20,$G$4:$G$203,G20,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U20" s="92"/>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="70"/>
@@ -3277,6 +3600,7 @@
       <x:c r="T21" s="60" t="str">
         <x:f>IF(COUNTA(A21:D21)+COUNTA(G21:S21)=0,"",IF(OR(A21="",B21="",C21="",D21="",G21="",H21="",J21="",R21=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A21)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B21)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B21,$G$4:$G$203,G21,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U21" s="91"/>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="A22" s="70"/>
@@ -3305,6 +3629,7 @@
       <x:c r="T22" s="60" t="str">
         <x:f>IF(COUNTA(A22:D22)+COUNTA(G22:S22)=0,"",IF(OR(A22="",B22="",C22="",D22="",G22="",H22="",J22="",R22=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A22)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B22)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B22,$G$4:$G$203,G22,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U22" s="92"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="70"/>
@@ -3333,6 +3658,7 @@
       <x:c r="T23" s="60" t="str">
         <x:f>IF(COUNTA(A23:D23)+COUNTA(G23:S23)=0,"",IF(OR(A23="",B23="",C23="",D23="",G23="",H23="",J23="",R23=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A23)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B23)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B23,$G$4:$G$203,G23,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U23" s="91"/>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="70"/>
@@ -3361,6 +3687,7 @@
       <x:c r="T24" s="60" t="str">
         <x:f>IF(COUNTA(A24:D24)+COUNTA(G24:S24)=0,"",IF(OR(A24="",B24="",C24="",D24="",G24="",H24="",J24="",R24=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A24)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B24)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B24,$G$4:$G$203,G24,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U24" s="92"/>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="A25" s="70"/>
@@ -3389,6 +3716,7 @@
       <x:c r="T25" s="60" t="str">
         <x:f>IF(COUNTA(A25:D25)+COUNTA(G25:S25)=0,"",IF(OR(A25="",B25="",C25="",D25="",G25="",H25="",J25="",R25=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A25)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B25)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B25,$G$4:$G$203,G25,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U25" s="91"/>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="A26" s="70"/>
@@ -3417,6 +3745,7 @@
       <x:c r="T26" s="60" t="str">
         <x:f>IF(COUNTA(A26:D26)+COUNTA(G26:S26)=0,"",IF(OR(A26="",B26="",C26="",D26="",G26="",H26="",J26="",R26=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A26)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B26)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B26,$G$4:$G$203,G26,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U26" s="92"/>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="A27" s="70"/>
@@ -3445,6 +3774,7 @@
       <x:c r="T27" s="60" t="str">
         <x:f>IF(COUNTA(A27:D27)+COUNTA(G27:S27)=0,"",IF(OR(A27="",B27="",C27="",D27="",G27="",H27="",J27="",R27=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A27)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B27)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B27,$G$4:$G$203,G27,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U27" s="91"/>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="A28" s="70"/>
@@ -3473,6 +3803,7 @@
       <x:c r="T28" s="60" t="str">
         <x:f>IF(COUNTA(A28:D28)+COUNTA(G28:S28)=0,"",IF(OR(A28="",B28="",C28="",D28="",G28="",H28="",J28="",R28=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A28)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B28)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B28,$G$4:$G$203,G28,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U28" s="92"/>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="A29" s="70"/>
@@ -3501,6 +3832,7 @@
       <x:c r="T29" s="60" t="str">
         <x:f>IF(COUNTA(A29:D29)+COUNTA(G29:S29)=0,"",IF(OR(A29="",B29="",C29="",D29="",G29="",H29="",J29="",R29=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A29)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B29)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B29,$G$4:$G$203,G29,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U29" s="91"/>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="A30" s="70"/>
@@ -3529,6 +3861,7 @@
       <x:c r="T30" s="60" t="str">
         <x:f>IF(COUNTA(A30:D30)+COUNTA(G30:S30)=0,"",IF(OR(A30="",B30="",C30="",D30="",G30="",H30="",J30="",R30=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A30)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B30)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B30,$G$4:$G$203,G30,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U30" s="92"/>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="A31" s="70"/>
@@ -3557,6 +3890,7 @@
       <x:c r="T31" s="60" t="str">
         <x:f>IF(COUNTA(A31:D31)+COUNTA(G31:S31)=0,"",IF(OR(A31="",B31="",C31="",D31="",G31="",H31="",J31="",R31=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A31)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B31)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B31,$G$4:$G$203,G31,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U31" s="91"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="A32" s="70"/>
@@ -3585,6 +3919,7 @@
       <x:c r="T32" s="60" t="str">
         <x:f>IF(COUNTA(A32:D32)+COUNTA(G32:S32)=0,"",IF(OR(A32="",B32="",C32="",D32="",G32="",H32="",J32="",R32=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A32)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B32)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B32,$G$4:$G$203,G32,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U32" s="92"/>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="A33" s="70"/>
@@ -3613,6 +3948,7 @@
       <x:c r="T33" s="60" t="str">
         <x:f>IF(COUNTA(A33:D33)+COUNTA(G33:S33)=0,"",IF(OR(A33="",B33="",C33="",D33="",G33="",H33="",J33="",R33=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A33)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B33)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B33,$G$4:$G$203,G33,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U33" s="91"/>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="A34" s="70"/>
@@ -3641,6 +3977,7 @@
       <x:c r="T34" s="60" t="str">
         <x:f>IF(COUNTA(A34:D34)+COUNTA(G34:S34)=0,"",IF(OR(A34="",B34="",C34="",D34="",G34="",H34="",J34="",R34=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A34)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B34)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B34,$G$4:$G$203,G34,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U34" s="92"/>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
       <x:c r="A35" s="70"/>
@@ -3669,6 +4006,7 @@
       <x:c r="T35" s="60" t="str">
         <x:f>IF(COUNTA(A35:D35)+COUNTA(G35:S35)=0,"",IF(OR(A35="",B35="",C35="",D35="",G35="",H35="",J35="",R35=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A35)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B35)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B35,$G$4:$G$203,G35,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U35" s="91"/>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
       <x:c r="A36" s="70"/>
@@ -3697,6 +4035,7 @@
       <x:c r="T36" s="60" t="str">
         <x:f>IF(COUNTA(A36:D36)+COUNTA(G36:S36)=0,"",IF(OR(A36="",B36="",C36="",D36="",G36="",H36="",J36="",R36=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A36)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B36)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B36,$G$4:$G$203,G36,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U36" s="92"/>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
       <x:c r="A37" s="70"/>
@@ -3725,6 +4064,7 @@
       <x:c r="T37" s="60" t="str">
         <x:f>IF(COUNTA(A37:D37)+COUNTA(G37:S37)=0,"",IF(OR(A37="",B37="",C37="",D37="",G37="",H37="",J37="",R37=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A37)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B37)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B37,$G$4:$G$203,G37,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U37" s="91"/>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
       <x:c r="A38" s="70"/>
@@ -3753,6 +4093,7 @@
       <x:c r="T38" s="60" t="str">
         <x:f>IF(COUNTA(A38:D38)+COUNTA(G38:S38)=0,"",IF(OR(A38="",B38="",C38="",D38="",G38="",H38="",J38="",R38=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A38)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B38)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B38,$G$4:$G$203,G38,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U38" s="92"/>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="70"/>
@@ -3781,6 +4122,7 @@
       <x:c r="T39" s="60" t="str">
         <x:f>IF(COUNTA(A39:D39)+COUNTA(G39:S39)=0,"",IF(OR(A39="",B39="",C39="",D39="",G39="",H39="",J39="",R39=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A39)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B39)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B39,$G$4:$G$203,G39,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U39" s="91"/>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
       <x:c r="A40" s="70"/>
@@ -3809,6 +4151,7 @@
       <x:c r="T40" s="60" t="str">
         <x:f>IF(COUNTA(A40:D40)+COUNTA(G40:S40)=0,"",IF(OR(A40="",B40="",C40="",D40="",G40="",H40="",J40="",R40=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A40)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B40)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B40,$G$4:$G$203,G40,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U40" s="92"/>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="70"/>
@@ -3837,6 +4180,7 @@
       <x:c r="T41" s="60" t="str">
         <x:f>IF(COUNTA(A41:D41)+COUNTA(G41:S41)=0,"",IF(OR(A41="",B41="",C41="",D41="",G41="",H41="",J41="",R41=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A41)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B41)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B41,$G$4:$G$203,G41,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U41" s="91"/>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
       <x:c r="A42" s="70"/>
@@ -3865,6 +4209,7 @@
       <x:c r="T42" s="60" t="str">
         <x:f>IF(COUNTA(A42:D42)+COUNTA(G42:S42)=0,"",IF(OR(A42="",B42="",C42="",D42="",G42="",H42="",J42="",R42=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A42)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B42)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B42,$G$4:$G$203,G42,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U42" s="92"/>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
       <x:c r="A43" s="70"/>
@@ -3893,6 +4238,7 @@
       <x:c r="T43" s="60" t="str">
         <x:f>IF(COUNTA(A43:D43)+COUNTA(G43:S43)=0,"",IF(OR(A43="",B43="",C43="",D43="",G43="",H43="",J43="",R43=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A43)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B43)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B43,$G$4:$G$203,G43,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U43" s="91"/>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
       <x:c r="A44" s="70"/>
@@ -3921,6 +4267,7 @@
       <x:c r="T44" s="60" t="str">
         <x:f>IF(COUNTA(A44:D44)+COUNTA(G44:S44)=0,"",IF(OR(A44="",B44="",C44="",D44="",G44="",H44="",J44="",R44=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A44)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B44)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B44,$G$4:$G$203,G44,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U44" s="92"/>
     </x:row>
     <x:row r="45" ht="22" customHeight="1">
       <x:c r="A45" s="70"/>
@@ -3949,6 +4296,7 @@
       <x:c r="T45" s="60" t="str">
         <x:f>IF(COUNTA(A45:D45)+COUNTA(G45:S45)=0,"",IF(OR(A45="",B45="",C45="",D45="",G45="",H45="",J45="",R45=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A45)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B45)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B45,$G$4:$G$203,G45,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U45" s="91"/>
     </x:row>
     <x:row r="46" ht="22" customHeight="1">
       <x:c r="A46" s="70"/>
@@ -3977,6 +4325,7 @@
       <x:c r="T46" s="60" t="str">
         <x:f>IF(COUNTA(A46:D46)+COUNTA(G46:S46)=0,"",IF(OR(A46="",B46="",C46="",D46="",G46="",H46="",J46="",R46=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A46)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B46)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B46,$G$4:$G$203,G46,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U46" s="92"/>
     </x:row>
     <x:row r="47" ht="22" customHeight="1">
       <x:c r="A47" s="70"/>
@@ -4005,6 +4354,7 @@
       <x:c r="T47" s="60" t="str">
         <x:f>IF(COUNTA(A47:D47)+COUNTA(G47:S47)=0,"",IF(OR(A47="",B47="",C47="",D47="",G47="",H47="",J47="",R47=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A47)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B47)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B47,$G$4:$G$203,G47,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U47" s="91"/>
     </x:row>
     <x:row r="48" ht="22" customHeight="1">
       <x:c r="A48" s="70"/>
@@ -4033,6 +4383,7 @@
       <x:c r="T48" s="60" t="str">
         <x:f>IF(COUNTA(A48:D48)+COUNTA(G48:S48)=0,"",IF(OR(A48="",B48="",C48="",D48="",G48="",H48="",J48="",R48=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A48)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B48)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B48,$G$4:$G$203,G48,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U48" s="92"/>
     </x:row>
     <x:row r="49" ht="22" customHeight="1">
       <x:c r="A49" s="70"/>
@@ -4061,6 +4412,7 @@
       <x:c r="T49" s="60" t="str">
         <x:f>IF(COUNTA(A49:D49)+COUNTA(G49:S49)=0,"",IF(OR(A49="",B49="",C49="",D49="",G49="",H49="",J49="",R49=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A49)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B49)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B49,$G$4:$G$203,G49,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U49" s="91"/>
     </x:row>
     <x:row r="50" ht="22" customHeight="1">
       <x:c r="A50" s="70"/>
@@ -4089,6 +4441,7 @@
       <x:c r="T50" s="60" t="str">
         <x:f>IF(COUNTA(A50:D50)+COUNTA(G50:S50)=0,"",IF(OR(A50="",B50="",C50="",D50="",G50="",H50="",J50="",R50=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A50)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B50)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B50,$G$4:$G$203,G50,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U50" s="92"/>
     </x:row>
     <x:row r="51" ht="22" customHeight="1">
       <x:c r="A51" s="70"/>
@@ -4117,6 +4470,7 @@
       <x:c r="T51" s="60" t="str">
         <x:f>IF(COUNTA(A51:D51)+COUNTA(G51:S51)=0,"",IF(OR(A51="",B51="",C51="",D51="",G51="",H51="",J51="",R51=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A51)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B51)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B51,$G$4:$G$203,G51,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U51" s="91"/>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
       <x:c r="A52" s="70"/>
@@ -4145,6 +4499,7 @@
       <x:c r="T52" s="60" t="str">
         <x:f>IF(COUNTA(A52:D52)+COUNTA(G52:S52)=0,"",IF(OR(A52="",B52="",C52="",D52="",G52="",H52="",J52="",R52=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A52)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B52)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B52,$G$4:$G$203,G52,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U52" s="92"/>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
       <x:c r="A53" s="70"/>
@@ -4173,6 +4528,7 @@
       <x:c r="T53" s="60" t="str">
         <x:f>IF(COUNTA(A53:D53)+COUNTA(G53:S53)=0,"",IF(OR(A53="",B53="",C53="",D53="",G53="",H53="",J53="",R53=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A53)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B53)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B53,$G$4:$G$203,G53,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U53" s="91"/>
     </x:row>
     <x:row r="54" ht="22" customHeight="1">
       <x:c r="A54" s="70"/>
@@ -4201,6 +4557,7 @@
       <x:c r="T54" s="60" t="str">
         <x:f>IF(COUNTA(A54:D54)+COUNTA(G54:S54)=0,"",IF(OR(A54="",B54="",C54="",D54="",G54="",H54="",J54="",R54=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A54)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B54)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B54,$G$4:$G$203,G54,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U54" s="92"/>
     </x:row>
     <x:row r="55" ht="22" customHeight="1">
       <x:c r="A55" s="70"/>
@@ -4229,6 +4586,7 @@
       <x:c r="T55" s="60" t="str">
         <x:f>IF(COUNTA(A55:D55)+COUNTA(G55:S55)=0,"",IF(OR(A55="",B55="",C55="",D55="",G55="",H55="",J55="",R55=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A55)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B55)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B55,$G$4:$G$203,G55,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U55" s="91"/>
     </x:row>
     <x:row r="56" ht="22" customHeight="1">
       <x:c r="A56" s="70"/>
@@ -4257,6 +4615,7 @@
       <x:c r="T56" s="60" t="str">
         <x:f>IF(COUNTA(A56:D56)+COUNTA(G56:S56)=0,"",IF(OR(A56="",B56="",C56="",D56="",G56="",H56="",J56="",R56=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A56)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B56)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B56,$G$4:$G$203,G56,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U56" s="92"/>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
       <x:c r="A57" s="70"/>
@@ -4285,6 +4644,7 @@
       <x:c r="T57" s="60" t="str">
         <x:f>IF(COUNTA(A57:D57)+COUNTA(G57:S57)=0,"",IF(OR(A57="",B57="",C57="",D57="",G57="",H57="",J57="",R57=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A57)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B57)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B57,$G$4:$G$203,G57,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U57" s="91"/>
     </x:row>
     <x:row r="58" ht="22" customHeight="1">
       <x:c r="A58" s="70"/>
@@ -4313,6 +4673,7 @@
       <x:c r="T58" s="60" t="str">
         <x:f>IF(COUNTA(A58:D58)+COUNTA(G58:S58)=0,"",IF(OR(A58="",B58="",C58="",D58="",G58="",H58="",J58="",R58=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A58)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B58)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B58,$G$4:$G$203,G58,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U58" s="92"/>
     </x:row>
     <x:row r="59" ht="22" customHeight="1">
       <x:c r="A59" s="70"/>
@@ -4341,6 +4702,7 @@
       <x:c r="T59" s="60" t="str">
         <x:f>IF(COUNTA(A59:D59)+COUNTA(G59:S59)=0,"",IF(OR(A59="",B59="",C59="",D59="",G59="",H59="",J59="",R59=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A59)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B59)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B59,$G$4:$G$203,G59,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U59" s="91"/>
     </x:row>
     <x:row r="60" ht="22" customHeight="1">
       <x:c r="A60" s="70"/>
@@ -4369,6 +4731,7 @@
       <x:c r="T60" s="60" t="str">
         <x:f>IF(COUNTA(A60:D60)+COUNTA(G60:S60)=0,"",IF(OR(A60="",B60="",C60="",D60="",G60="",H60="",J60="",R60=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A60)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B60)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B60,$G$4:$G$203,G60,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U60" s="92"/>
     </x:row>
     <x:row r="61" ht="22" customHeight="1">
       <x:c r="A61" s="70"/>
@@ -4397,6 +4760,7 @@
       <x:c r="T61" s="60" t="str">
         <x:f>IF(COUNTA(A61:D61)+COUNTA(G61:S61)=0,"",IF(OR(A61="",B61="",C61="",D61="",G61="",H61="",J61="",R61=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A61)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B61)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B61,$G$4:$G$203,G61,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U61" s="91"/>
     </x:row>
     <x:row r="62" ht="22" customHeight="1">
       <x:c r="A62" s="70"/>
@@ -4425,6 +4789,7 @@
       <x:c r="T62" s="60" t="str">
         <x:f>IF(COUNTA(A62:D62)+COUNTA(G62:S62)=0,"",IF(OR(A62="",B62="",C62="",D62="",G62="",H62="",J62="",R62=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A62)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B62)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B62,$G$4:$G$203,G62,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U62" s="92"/>
     </x:row>
     <x:row r="63" ht="22" customHeight="1">
       <x:c r="A63" s="70"/>
@@ -4453,6 +4818,7 @@
       <x:c r="T63" s="60" t="str">
         <x:f>IF(COUNTA(A63:D63)+COUNTA(G63:S63)=0,"",IF(OR(A63="",B63="",C63="",D63="",G63="",H63="",J63="",R63=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A63)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B63)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B63,$G$4:$G$203,G63,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U63" s="91"/>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="70"/>
@@ -4481,6 +4847,7 @@
       <x:c r="T64" s="60" t="str">
         <x:f>IF(COUNTA(A64:D64)+COUNTA(G64:S64)=0,"",IF(OR(A64="",B64="",C64="",D64="",G64="",H64="",J64="",R64=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A64)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B64)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B64,$G$4:$G$203,G64,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U64" s="92"/>
     </x:row>
     <x:row r="65" ht="22" customHeight="1">
       <x:c r="A65" s="70"/>
@@ -4509,6 +4876,7 @@
       <x:c r="T65" s="60" t="str">
         <x:f>IF(COUNTA(A65:D65)+COUNTA(G65:S65)=0,"",IF(OR(A65="",B65="",C65="",D65="",G65="",H65="",J65="",R65=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A65)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B65)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B65,$G$4:$G$203,G65,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U65" s="91"/>
     </x:row>
     <x:row r="66" ht="22" customHeight="1">
       <x:c r="A66" s="70"/>
@@ -4537,6 +4905,7 @@
       <x:c r="T66" s="60" t="str">
         <x:f>IF(COUNTA(A66:D66)+COUNTA(G66:S66)=0,"",IF(OR(A66="",B66="",C66="",D66="",G66="",H66="",J66="",R66=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A66)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B66)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B66,$G$4:$G$203,G66,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U66" s="92"/>
     </x:row>
     <x:row r="67" ht="22" customHeight="1">
       <x:c r="A67" s="70"/>
@@ -4565,6 +4934,7 @@
       <x:c r="T67" s="60" t="str">
         <x:f>IF(COUNTA(A67:D67)+COUNTA(G67:S67)=0,"",IF(OR(A67="",B67="",C67="",D67="",G67="",H67="",J67="",R67=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A67)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B67)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B67,$G$4:$G$203,G67,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U67" s="91"/>
     </x:row>
     <x:row r="68" ht="22" customHeight="1">
       <x:c r="A68" s="70"/>
@@ -4593,6 +4963,7 @@
       <x:c r="T68" s="60" t="str">
         <x:f>IF(COUNTA(A68:D68)+COUNTA(G68:S68)=0,"",IF(OR(A68="",B68="",C68="",D68="",G68="",H68="",J68="",R68=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A68)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B68)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B68,$G$4:$G$203,G68,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U68" s="92"/>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
       <x:c r="A69" s="70"/>
@@ -4621,6 +4992,7 @@
       <x:c r="T69" s="60" t="str">
         <x:f>IF(COUNTA(A69:D69)+COUNTA(G69:S69)=0,"",IF(OR(A69="",B69="",C69="",D69="",G69="",H69="",J69="",R69=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A69)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B69)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B69,$G$4:$G$203,G69,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U69" s="91"/>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
       <x:c r="A70" s="70"/>
@@ -4649,6 +5021,7 @@
       <x:c r="T70" s="60" t="str">
         <x:f>IF(COUNTA(A70:D70)+COUNTA(G70:S70)=0,"",IF(OR(A70="",B70="",C70="",D70="",G70="",H70="",J70="",R70=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A70)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B70)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B70,$G$4:$G$203,G70,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U70" s="92"/>
     </x:row>
     <x:row r="71" ht="22" customHeight="1">
       <x:c r="A71" s="70"/>
@@ -4677,6 +5050,7 @@
       <x:c r="T71" s="60" t="str">
         <x:f>IF(COUNTA(A71:D71)+COUNTA(G71:S71)=0,"",IF(OR(A71="",B71="",C71="",D71="",G71="",H71="",J71="",R71=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A71)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B71)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B71,$G$4:$G$203,G71,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U71" s="91"/>
     </x:row>
     <x:row r="72" ht="22" customHeight="1">
       <x:c r="A72" s="70"/>
@@ -4705,6 +5079,7 @@
       <x:c r="T72" s="60" t="str">
         <x:f>IF(COUNTA(A72:D72)+COUNTA(G72:S72)=0,"",IF(OR(A72="",B72="",C72="",D72="",G72="",H72="",J72="",R72=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A72)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B72)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B72,$G$4:$G$203,G72,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U72" s="92"/>
     </x:row>
     <x:row r="73" ht="22" customHeight="1">
       <x:c r="A73" s="70"/>
@@ -4733,6 +5108,7 @@
       <x:c r="T73" s="60" t="str">
         <x:f>IF(COUNTA(A73:D73)+COUNTA(G73:S73)=0,"",IF(OR(A73="",B73="",C73="",D73="",G73="",H73="",J73="",R73=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A73)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B73)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B73,$G$4:$G$203,G73,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U73" s="91"/>
     </x:row>
     <x:row r="74" ht="22" customHeight="1">
       <x:c r="A74" s="70"/>
@@ -4761,6 +5137,7 @@
       <x:c r="T74" s="60" t="str">
         <x:f>IF(COUNTA(A74:D74)+COUNTA(G74:S74)=0,"",IF(OR(A74="",B74="",C74="",D74="",G74="",H74="",J74="",R74=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A74)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B74)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B74,$G$4:$G$203,G74,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U74" s="92"/>
     </x:row>
     <x:row r="75" ht="22" customHeight="1">
       <x:c r="A75" s="70"/>
@@ -4789,6 +5166,7 @@
       <x:c r="T75" s="60" t="str">
         <x:f>IF(COUNTA(A75:D75)+COUNTA(G75:S75)=0,"",IF(OR(A75="",B75="",C75="",D75="",G75="",H75="",J75="",R75=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A75)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B75)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B75,$G$4:$G$203,G75,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U75" s="91"/>
     </x:row>
     <x:row r="76" ht="22" customHeight="1">
       <x:c r="A76" s="70"/>
@@ -4817,6 +5195,7 @@
       <x:c r="T76" s="60" t="str">
         <x:f>IF(COUNTA(A76:D76)+COUNTA(G76:S76)=0,"",IF(OR(A76="",B76="",C76="",D76="",G76="",H76="",J76="",R76=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A76)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B76)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B76,$G$4:$G$203,G76,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U76" s="92"/>
     </x:row>
     <x:row r="77" ht="22" customHeight="1">
       <x:c r="A77" s="70"/>
@@ -4845,6 +5224,7 @@
       <x:c r="T77" s="60" t="str">
         <x:f>IF(COUNTA(A77:D77)+COUNTA(G77:S77)=0,"",IF(OR(A77="",B77="",C77="",D77="",G77="",H77="",J77="",R77=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A77)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B77)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B77,$G$4:$G$203,G77,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U77" s="91"/>
     </x:row>
     <x:row r="78" ht="22" customHeight="1">
       <x:c r="A78" s="70"/>
@@ -4873,6 +5253,7 @@
       <x:c r="T78" s="60" t="str">
         <x:f>IF(COUNTA(A78:D78)+COUNTA(G78:S78)=0,"",IF(OR(A78="",B78="",C78="",D78="",G78="",H78="",J78="",R78=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A78)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B78)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B78,$G$4:$G$203,G78,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U78" s="92"/>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
       <x:c r="A79" s="70"/>
@@ -4901,6 +5282,7 @@
       <x:c r="T79" s="60" t="str">
         <x:f>IF(COUNTA(A79:D79)+COUNTA(G79:S79)=0,"",IF(OR(A79="",B79="",C79="",D79="",G79="",H79="",J79="",R79=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A79)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B79)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B79,$G$4:$G$203,G79,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U79" s="91"/>
     </x:row>
     <x:row r="80" ht="22" customHeight="1">
       <x:c r="A80" s="70"/>
@@ -4929,6 +5311,7 @@
       <x:c r="T80" s="60" t="str">
         <x:f>IF(COUNTA(A80:D80)+COUNTA(G80:S80)=0,"",IF(OR(A80="",B80="",C80="",D80="",G80="",H80="",J80="",R80=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A80)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B80)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B80,$G$4:$G$203,G80,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U80" s="92"/>
     </x:row>
     <x:row r="81" ht="22" customHeight="1">
       <x:c r="A81" s="70"/>
@@ -4957,6 +5340,7 @@
       <x:c r="T81" s="60" t="str">
         <x:f>IF(COUNTA(A81:D81)+COUNTA(G81:S81)=0,"",IF(OR(A81="",B81="",C81="",D81="",G81="",H81="",J81="",R81=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A81)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B81)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B81,$G$4:$G$203,G81,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U81" s="91"/>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
       <x:c r="A82" s="70"/>
@@ -4985,6 +5369,7 @@
       <x:c r="T82" s="60" t="str">
         <x:f>IF(COUNTA(A82:D82)+COUNTA(G82:S82)=0,"",IF(OR(A82="",B82="",C82="",D82="",G82="",H82="",J82="",R82=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A82)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B82)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B82,$G$4:$G$203,G82,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U82" s="92"/>
     </x:row>
     <x:row r="83" ht="22" customHeight="1">
       <x:c r="A83" s="70"/>
@@ -5013,6 +5398,7 @@
       <x:c r="T83" s="60" t="str">
         <x:f>IF(COUNTA(A83:D83)+COUNTA(G83:S83)=0,"",IF(OR(A83="",B83="",C83="",D83="",G83="",H83="",J83="",R83=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A83)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B83)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B83,$G$4:$G$203,G83,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U83" s="91"/>
     </x:row>
     <x:row r="84" ht="22" customHeight="1">
       <x:c r="A84" s="70"/>
@@ -5041,6 +5427,7 @@
       <x:c r="T84" s="60" t="str">
         <x:f>IF(COUNTA(A84:D84)+COUNTA(G84:S84)=0,"",IF(OR(A84="",B84="",C84="",D84="",G84="",H84="",J84="",R84=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A84)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B84)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B84,$G$4:$G$203,G84,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U84" s="92"/>
     </x:row>
     <x:row r="85" ht="22" customHeight="1">
       <x:c r="A85" s="70"/>
@@ -5069,6 +5456,7 @@
       <x:c r="T85" s="60" t="str">
         <x:f>IF(COUNTA(A85:D85)+COUNTA(G85:S85)=0,"",IF(OR(A85="",B85="",C85="",D85="",G85="",H85="",J85="",R85=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A85)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B85)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B85,$G$4:$G$203,G85,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U85" s="91"/>
     </x:row>
     <x:row r="86" ht="22" customHeight="1">
       <x:c r="A86" s="70"/>
@@ -5097,6 +5485,7 @@
       <x:c r="T86" s="60" t="str">
         <x:f>IF(COUNTA(A86:D86)+COUNTA(G86:S86)=0,"",IF(OR(A86="",B86="",C86="",D86="",G86="",H86="",J86="",R86=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A86)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B86)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B86,$G$4:$G$203,G86,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U86" s="92"/>
     </x:row>
     <x:row r="87" ht="22" customHeight="1">
       <x:c r="A87" s="70"/>
@@ -5125,6 +5514,7 @@
       <x:c r="T87" s="60" t="str">
         <x:f>IF(COUNTA(A87:D87)+COUNTA(G87:S87)=0,"",IF(OR(A87="",B87="",C87="",D87="",G87="",H87="",J87="",R87=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A87)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B87)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B87,$G$4:$G$203,G87,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U87" s="91"/>
     </x:row>
     <x:row r="88" ht="22" customHeight="1">
       <x:c r="A88" s="70"/>
@@ -5153,6 +5543,7 @@
       <x:c r="T88" s="60" t="str">
         <x:f>IF(COUNTA(A88:D88)+COUNTA(G88:S88)=0,"",IF(OR(A88="",B88="",C88="",D88="",G88="",H88="",J88="",R88=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A88)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B88)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B88,$G$4:$G$203,G88,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U88" s="92"/>
     </x:row>
     <x:row r="89" ht="22" customHeight="1">
       <x:c r="A89" s="70"/>
@@ -5181,6 +5572,7 @@
       <x:c r="T89" s="60" t="str">
         <x:f>IF(COUNTA(A89:D89)+COUNTA(G89:S89)=0,"",IF(OR(A89="",B89="",C89="",D89="",G89="",H89="",J89="",R89=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A89)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B89)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B89,$G$4:$G$203,G89,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U89" s="91"/>
     </x:row>
     <x:row r="90" ht="22" customHeight="1">
       <x:c r="A90" s="70"/>
@@ -5209,6 +5601,7 @@
       <x:c r="T90" s="60" t="str">
         <x:f>IF(COUNTA(A90:D90)+COUNTA(G90:S90)=0,"",IF(OR(A90="",B90="",C90="",D90="",G90="",H90="",J90="",R90=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A90)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B90)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B90,$G$4:$G$203,G90,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U90" s="92"/>
     </x:row>
     <x:row r="91" ht="22" customHeight="1">
       <x:c r="A91" s="70"/>
@@ -5237,6 +5630,7 @@
       <x:c r="T91" s="60" t="str">
         <x:f>IF(COUNTA(A91:D91)+COUNTA(G91:S91)=0,"",IF(OR(A91="",B91="",C91="",D91="",G91="",H91="",J91="",R91=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A91)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B91)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B91,$G$4:$G$203,G91,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U91" s="91"/>
     </x:row>
     <x:row r="92" ht="22" customHeight="1">
       <x:c r="A92" s="70"/>
@@ -5265,6 +5659,7 @@
       <x:c r="T92" s="60" t="str">
         <x:f>IF(COUNTA(A92:D92)+COUNTA(G92:S92)=0,"",IF(OR(A92="",B92="",C92="",D92="",G92="",H92="",J92="",R92=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A92)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B92)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B92,$G$4:$G$203,G92,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U92" s="92"/>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
       <x:c r="A93" s="70"/>
@@ -5293,6 +5688,7 @@
       <x:c r="T93" s="60" t="str">
         <x:f>IF(COUNTA(A93:D93)+COUNTA(G93:S93)=0,"",IF(OR(A93="",B93="",C93="",D93="",G93="",H93="",J93="",R93=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A93)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B93)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B93,$G$4:$G$203,G93,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U93" s="91"/>
     </x:row>
     <x:row r="94" ht="22" customHeight="1">
       <x:c r="A94" s="70"/>
@@ -5321,6 +5717,7 @@
       <x:c r="T94" s="60" t="str">
         <x:f>IF(COUNTA(A94:D94)+COUNTA(G94:S94)=0,"",IF(OR(A94="",B94="",C94="",D94="",G94="",H94="",J94="",R94=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A94)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B94)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B94,$G$4:$G$203,G94,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U94" s="92"/>
     </x:row>
     <x:row r="95" ht="22" customHeight="1">
       <x:c r="A95" s="70"/>
@@ -5349,6 +5746,7 @@
       <x:c r="T95" s="60" t="str">
         <x:f>IF(COUNTA(A95:D95)+COUNTA(G95:S95)=0,"",IF(OR(A95="",B95="",C95="",D95="",G95="",H95="",J95="",R95=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A95)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B95)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B95,$G$4:$G$203,G95,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U95" s="91"/>
     </x:row>
     <x:row r="96" ht="22" customHeight="1">
       <x:c r="A96" s="70"/>
@@ -5377,6 +5775,7 @@
       <x:c r="T96" s="60" t="str">
         <x:f>IF(COUNTA(A96:D96)+COUNTA(G96:S96)=0,"",IF(OR(A96="",B96="",C96="",D96="",G96="",H96="",J96="",R96=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A96)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B96)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B96,$G$4:$G$203,G96,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U96" s="92"/>
     </x:row>
     <x:row r="97" ht="22" customHeight="1">
       <x:c r="A97" s="70"/>
@@ -5405,6 +5804,7 @@
       <x:c r="T97" s="60" t="str">
         <x:f>IF(COUNTA(A97:D97)+COUNTA(G97:S97)=0,"",IF(OR(A97="",B97="",C97="",D97="",G97="",H97="",J97="",R97=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A97)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B97)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B97,$G$4:$G$203,G97,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U97" s="91"/>
     </x:row>
     <x:row r="98" ht="22" customHeight="1">
       <x:c r="A98" s="70"/>
@@ -5433,6 +5833,7 @@
       <x:c r="T98" s="60" t="str">
         <x:f>IF(COUNTA(A98:D98)+COUNTA(G98:S98)=0,"",IF(OR(A98="",B98="",C98="",D98="",G98="",H98="",J98="",R98=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A98)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B98)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B98,$G$4:$G$203,G98,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U98" s="92"/>
     </x:row>
     <x:row r="99" ht="22" customHeight="1">
       <x:c r="A99" s="70"/>
@@ -5461,6 +5862,7 @@
       <x:c r="T99" s="60" t="str">
         <x:f>IF(COUNTA(A99:D99)+COUNTA(G99:S99)=0,"",IF(OR(A99="",B99="",C99="",D99="",G99="",H99="",J99="",R99=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A99)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B99)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B99,$G$4:$G$203,G99,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U99" s="91"/>
     </x:row>
     <x:row r="100" ht="22" customHeight="1">
       <x:c r="A100" s="70"/>
@@ -5489,6 +5891,7 @@
       <x:c r="T100" s="60" t="str">
         <x:f>IF(COUNTA(A100:D100)+COUNTA(G100:S100)=0,"",IF(OR(A100="",B100="",C100="",D100="",G100="",H100="",J100="",R100=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A100)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B100)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B100,$G$4:$G$203,G100,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U100" s="92"/>
     </x:row>
     <x:row r="101" ht="22" customHeight="1">
       <x:c r="A101" s="70"/>
@@ -5517,6 +5920,7 @@
       <x:c r="T101" s="60" t="str">
         <x:f>IF(COUNTA(A101:D101)+COUNTA(G101:S101)=0,"",IF(OR(A101="",B101="",C101="",D101="",G101="",H101="",J101="",R101=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A101)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B101)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B101,$G$4:$G$203,G101,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U101" s="91"/>
     </x:row>
     <x:row r="102" ht="22" customHeight="1">
       <x:c r="A102" s="70"/>
@@ -5545,6 +5949,7 @@
       <x:c r="T102" s="60" t="str">
         <x:f>IF(COUNTA(A102:D102)+COUNTA(G102:S102)=0,"",IF(OR(A102="",B102="",C102="",D102="",G102="",H102="",J102="",R102=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A102)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B102)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B102,$G$4:$G$203,G102,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U102" s="92"/>
     </x:row>
     <x:row r="103" ht="22" customHeight="1">
       <x:c r="A103" s="70"/>
@@ -5573,6 +5978,7 @@
       <x:c r="T103" s="60" t="str">
         <x:f>IF(COUNTA(A103:D103)+COUNTA(G103:S103)=0,"",IF(OR(A103="",B103="",C103="",D103="",G103="",H103="",J103="",R103=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A103)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B103)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B103,$G$4:$G$203,G103,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U103" s="91"/>
     </x:row>
     <x:row r="104" ht="22" customHeight="1">
       <x:c r="A104" s="70"/>
@@ -5601,6 +6007,7 @@
       <x:c r="T104" s="60" t="str">
         <x:f>IF(COUNTA(A104:D104)+COUNTA(G104:S104)=0,"",IF(OR(A104="",B104="",C104="",D104="",G104="",H104="",J104="",R104=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A104)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B104)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B104,$G$4:$G$203,G104,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U104" s="92"/>
     </x:row>
     <x:row r="105" ht="22" customHeight="1">
       <x:c r="A105" s="70"/>
@@ -5629,6 +6036,7 @@
       <x:c r="T105" s="60" t="str">
         <x:f>IF(COUNTA(A105:D105)+COUNTA(G105:S105)=0,"",IF(OR(A105="",B105="",C105="",D105="",G105="",H105="",J105="",R105=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A105)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B105)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B105,$G$4:$G$203,G105,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U105" s="91"/>
     </x:row>
     <x:row r="106" ht="22" customHeight="1">
       <x:c r="A106" s="70"/>
@@ -5657,6 +6065,7 @@
       <x:c r="T106" s="60" t="str">
         <x:f>IF(COUNTA(A106:D106)+COUNTA(G106:S106)=0,"",IF(OR(A106="",B106="",C106="",D106="",G106="",H106="",J106="",R106=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A106)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B106)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B106,$G$4:$G$203,G106,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U106" s="92"/>
     </x:row>
     <x:row r="107" ht="22" customHeight="1">
       <x:c r="A107" s="70"/>
@@ -5685,6 +6094,7 @@
       <x:c r="T107" s="60" t="str">
         <x:f>IF(COUNTA(A107:D107)+COUNTA(G107:S107)=0,"",IF(OR(A107="",B107="",C107="",D107="",G107="",H107="",J107="",R107=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A107)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B107)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B107,$G$4:$G$203,G107,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U107" s="91"/>
     </x:row>
     <x:row r="108" ht="22" customHeight="1">
       <x:c r="A108" s="70"/>
@@ -5713,6 +6123,7 @@
       <x:c r="T108" s="60" t="str">
         <x:f>IF(COUNTA(A108:D108)+COUNTA(G108:S108)=0,"",IF(OR(A108="",B108="",C108="",D108="",G108="",H108="",J108="",R108=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A108)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B108)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B108,$G$4:$G$203,G108,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U108" s="92"/>
     </x:row>
     <x:row r="109" ht="22" customHeight="1">
       <x:c r="A109" s="70"/>
@@ -5741,6 +6152,7 @@
       <x:c r="T109" s="60" t="str">
         <x:f>IF(COUNTA(A109:D109)+COUNTA(G109:S109)=0,"",IF(OR(A109="",B109="",C109="",D109="",G109="",H109="",J109="",R109=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A109)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B109)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B109,$G$4:$G$203,G109,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U109" s="91"/>
     </x:row>
     <x:row r="110" ht="22" customHeight="1">
       <x:c r="A110" s="70"/>
@@ -5769,6 +6181,7 @@
       <x:c r="T110" s="60" t="str">
         <x:f>IF(COUNTA(A110:D110)+COUNTA(G110:S110)=0,"",IF(OR(A110="",B110="",C110="",D110="",G110="",H110="",J110="",R110=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A110)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B110)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B110,$G$4:$G$203,G110,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U110" s="92"/>
     </x:row>
     <x:row r="111" ht="22" customHeight="1">
       <x:c r="A111" s="70"/>
@@ -5797,6 +6210,7 @@
       <x:c r="T111" s="60" t="str">
         <x:f>IF(COUNTA(A111:D111)+COUNTA(G111:S111)=0,"",IF(OR(A111="",B111="",C111="",D111="",G111="",H111="",J111="",R111=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A111)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B111)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B111,$G$4:$G$203,G111,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U111" s="91"/>
     </x:row>
     <x:row r="112" ht="22" customHeight="1">
       <x:c r="A112" s="70"/>
@@ -5825,6 +6239,7 @@
       <x:c r="T112" s="60" t="str">
         <x:f>IF(COUNTA(A112:D112)+COUNTA(G112:S112)=0,"",IF(OR(A112="",B112="",C112="",D112="",G112="",H112="",J112="",R112=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A112)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B112)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B112,$G$4:$G$203,G112,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U112" s="92"/>
     </x:row>
     <x:row r="113" ht="22" customHeight="1">
       <x:c r="A113" s="70"/>
@@ -5853,6 +6268,7 @@
       <x:c r="T113" s="60" t="str">
         <x:f>IF(COUNTA(A113:D113)+COUNTA(G113:S113)=0,"",IF(OR(A113="",B113="",C113="",D113="",G113="",H113="",J113="",R113=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A113)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B113)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B113,$G$4:$G$203,G113,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U113" s="91"/>
     </x:row>
     <x:row r="114" ht="22" customHeight="1">
       <x:c r="A114" s="70"/>
@@ -5881,6 +6297,7 @@
       <x:c r="T114" s="60" t="str">
         <x:f>IF(COUNTA(A114:D114)+COUNTA(G114:S114)=0,"",IF(OR(A114="",B114="",C114="",D114="",G114="",H114="",J114="",R114=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A114)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B114)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B114,$G$4:$G$203,G114,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U114" s="92"/>
     </x:row>
     <x:row r="115" ht="22" customHeight="1">
       <x:c r="A115" s="70"/>
@@ -5909,6 +6326,7 @@
       <x:c r="T115" s="60" t="str">
         <x:f>IF(COUNTA(A115:D115)+COUNTA(G115:S115)=0,"",IF(OR(A115="",B115="",C115="",D115="",G115="",H115="",J115="",R115=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A115)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B115)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B115,$G$4:$G$203,G115,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U115" s="91"/>
     </x:row>
     <x:row r="116" ht="22" customHeight="1">
       <x:c r="A116" s="70"/>
@@ -5937,6 +6355,7 @@
       <x:c r="T116" s="60" t="str">
         <x:f>IF(COUNTA(A116:D116)+COUNTA(G116:S116)=0,"",IF(OR(A116="",B116="",C116="",D116="",G116="",H116="",J116="",R116=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A116)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B116)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B116,$G$4:$G$203,G116,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U116" s="92"/>
     </x:row>
     <x:row r="117" ht="22" customHeight="1">
       <x:c r="A117" s="70"/>
@@ -5965,6 +6384,7 @@
       <x:c r="T117" s="60" t="str">
         <x:f>IF(COUNTA(A117:D117)+COUNTA(G117:S117)=0,"",IF(OR(A117="",B117="",C117="",D117="",G117="",H117="",J117="",R117=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A117)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B117)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B117,$G$4:$G$203,G117,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U117" s="91"/>
     </x:row>
     <x:row r="118" ht="22" customHeight="1">
       <x:c r="A118" s="70"/>
@@ -5993,6 +6413,7 @@
       <x:c r="T118" s="60" t="str">
         <x:f>IF(COUNTA(A118:D118)+COUNTA(G118:S118)=0,"",IF(OR(A118="",B118="",C118="",D118="",G118="",H118="",J118="",R118=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A118)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B118)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B118,$G$4:$G$203,G118,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U118" s="92"/>
     </x:row>
     <x:row r="119" ht="22" customHeight="1">
       <x:c r="A119" s="70"/>
@@ -6021,6 +6442,7 @@
       <x:c r="T119" s="60" t="str">
         <x:f>IF(COUNTA(A119:D119)+COUNTA(G119:S119)=0,"",IF(OR(A119="",B119="",C119="",D119="",G119="",H119="",J119="",R119=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A119)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B119)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B119,$G$4:$G$203,G119,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U119" s="91"/>
     </x:row>
     <x:row r="120" ht="22" customHeight="1">
       <x:c r="A120" s="70"/>
@@ -6049,6 +6471,7 @@
       <x:c r="T120" s="60" t="str">
         <x:f>IF(COUNTA(A120:D120)+COUNTA(G120:S120)=0,"",IF(OR(A120="",B120="",C120="",D120="",G120="",H120="",J120="",R120=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A120)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B120)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B120,$G$4:$G$203,G120,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U120" s="92"/>
     </x:row>
     <x:row r="121" ht="22" customHeight="1">
       <x:c r="A121" s="70"/>
@@ -6077,6 +6500,7 @@
       <x:c r="T121" s="60" t="str">
         <x:f>IF(COUNTA(A121:D121)+COUNTA(G121:S121)=0,"",IF(OR(A121="",B121="",C121="",D121="",G121="",H121="",J121="",R121=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A121)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B121)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B121,$G$4:$G$203,G121,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U121" s="91"/>
     </x:row>
     <x:row r="122" ht="22" customHeight="1">
       <x:c r="A122" s="70"/>
@@ -6105,6 +6529,7 @@
       <x:c r="T122" s="60" t="str">
         <x:f>IF(COUNTA(A122:D122)+COUNTA(G122:S122)=0,"",IF(OR(A122="",B122="",C122="",D122="",G122="",H122="",J122="",R122=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A122)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B122)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B122,$G$4:$G$203,G122,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U122" s="92"/>
     </x:row>
     <x:row r="123" ht="22" customHeight="1">
       <x:c r="A123" s="70"/>
@@ -6133,6 +6558,7 @@
       <x:c r="T123" s="60" t="str">
         <x:f>IF(COUNTA(A123:D123)+COUNTA(G123:S123)=0,"",IF(OR(A123="",B123="",C123="",D123="",G123="",H123="",J123="",R123=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A123)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B123)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B123,$G$4:$G$203,G123,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U123" s="91"/>
     </x:row>
     <x:row r="124" ht="22" customHeight="1">
       <x:c r="A124" s="70"/>
@@ -6161,6 +6587,7 @@
       <x:c r="T124" s="60" t="str">
         <x:f>IF(COUNTA(A124:D124)+COUNTA(G124:S124)=0,"",IF(OR(A124="",B124="",C124="",D124="",G124="",H124="",J124="",R124=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A124)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B124)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B124,$G$4:$G$203,G124,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U124" s="92"/>
     </x:row>
     <x:row r="125" ht="22" customHeight="1">
       <x:c r="A125" s="70"/>
@@ -6189,6 +6616,7 @@
       <x:c r="T125" s="60" t="str">
         <x:f>IF(COUNTA(A125:D125)+COUNTA(G125:S125)=0,"",IF(OR(A125="",B125="",C125="",D125="",G125="",H125="",J125="",R125=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A125)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B125)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B125,$G$4:$G$203,G125,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U125" s="91"/>
     </x:row>
     <x:row r="126" ht="22" customHeight="1">
       <x:c r="A126" s="70"/>
@@ -6217,6 +6645,7 @@
       <x:c r="T126" s="60" t="str">
         <x:f>IF(COUNTA(A126:D126)+COUNTA(G126:S126)=0,"",IF(OR(A126="",B126="",C126="",D126="",G126="",H126="",J126="",R126=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A126)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B126)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B126,$G$4:$G$203,G126,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U126" s="92"/>
     </x:row>
     <x:row r="127" ht="22" customHeight="1">
       <x:c r="A127" s="70"/>
@@ -6245,6 +6674,7 @@
       <x:c r="T127" s="60" t="str">
         <x:f>IF(COUNTA(A127:D127)+COUNTA(G127:S127)=0,"",IF(OR(A127="",B127="",C127="",D127="",G127="",H127="",J127="",R127=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A127)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B127)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B127,$G$4:$G$203,G127,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U127" s="91"/>
     </x:row>
     <x:row r="128" ht="22" customHeight="1">
       <x:c r="A128" s="70"/>
@@ -6273,6 +6703,7 @@
       <x:c r="T128" s="60" t="str">
         <x:f>IF(COUNTA(A128:D128)+COUNTA(G128:S128)=0,"",IF(OR(A128="",B128="",C128="",D128="",G128="",H128="",J128="",R128=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A128)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B128)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B128,$G$4:$G$203,G128,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U128" s="92"/>
     </x:row>
     <x:row r="129" ht="22" customHeight="1">
       <x:c r="A129" s="70"/>
@@ -6301,6 +6732,7 @@
       <x:c r="T129" s="60" t="str">
         <x:f>IF(COUNTA(A129:D129)+COUNTA(G129:S129)=0,"",IF(OR(A129="",B129="",C129="",D129="",G129="",H129="",J129="",R129=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A129)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B129)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B129,$G$4:$G$203,G129,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U129" s="91"/>
     </x:row>
     <x:row r="130" ht="22" customHeight="1">
       <x:c r="A130" s="70"/>
@@ -6329,6 +6761,7 @@
       <x:c r="T130" s="60" t="str">
         <x:f>IF(COUNTA(A130:D130)+COUNTA(G130:S130)=0,"",IF(OR(A130="",B130="",C130="",D130="",G130="",H130="",J130="",R130=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A130)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B130)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B130,$G$4:$G$203,G130,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U130" s="92"/>
     </x:row>
     <x:row r="131" ht="22" customHeight="1">
       <x:c r="A131" s="70"/>
@@ -6357,6 +6790,7 @@
       <x:c r="T131" s="60" t="str">
         <x:f>IF(COUNTA(A131:D131)+COUNTA(G131:S131)=0,"",IF(OR(A131="",B131="",C131="",D131="",G131="",H131="",J131="",R131=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A131)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B131)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B131,$G$4:$G$203,G131,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U131" s="91"/>
     </x:row>
     <x:row r="132" ht="22" customHeight="1">
       <x:c r="A132" s="70"/>
@@ -6385,6 +6819,7 @@
       <x:c r="T132" s="60" t="str">
         <x:f>IF(COUNTA(A132:D132)+COUNTA(G132:S132)=0,"",IF(OR(A132="",B132="",C132="",D132="",G132="",H132="",J132="",R132=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A132)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B132)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B132,$G$4:$G$203,G132,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U132" s="92"/>
     </x:row>
     <x:row r="133" ht="22" customHeight="1">
       <x:c r="A133" s="70"/>
@@ -6413,6 +6848,7 @@
       <x:c r="T133" s="60" t="str">
         <x:f>IF(COUNTA(A133:D133)+COUNTA(G133:S133)=0,"",IF(OR(A133="",B133="",C133="",D133="",G133="",H133="",J133="",R133=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A133)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B133)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B133,$G$4:$G$203,G133,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U133" s="91"/>
     </x:row>
     <x:row r="134" ht="22" customHeight="1">
       <x:c r="A134" s="70"/>
@@ -6441,6 +6877,7 @@
       <x:c r="T134" s="60" t="str">
         <x:f>IF(COUNTA(A134:D134)+COUNTA(G134:S134)=0,"",IF(OR(A134="",B134="",C134="",D134="",G134="",H134="",J134="",R134=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A134)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B134)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B134,$G$4:$G$203,G134,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U134" s="92"/>
     </x:row>
     <x:row r="135" ht="22" customHeight="1">
       <x:c r="A135" s="70"/>
@@ -6469,6 +6906,7 @@
       <x:c r="T135" s="60" t="str">
         <x:f>IF(COUNTA(A135:D135)+COUNTA(G135:S135)=0,"",IF(OR(A135="",B135="",C135="",D135="",G135="",H135="",J135="",R135=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A135)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B135)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B135,$G$4:$G$203,G135,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U135" s="91"/>
     </x:row>
     <x:row r="136" ht="22" customHeight="1">
       <x:c r="A136" s="70"/>
@@ -6497,6 +6935,7 @@
       <x:c r="T136" s="60" t="str">
         <x:f>IF(COUNTA(A136:D136)+COUNTA(G136:S136)=0,"",IF(OR(A136="",B136="",C136="",D136="",G136="",H136="",J136="",R136=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A136)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B136)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B136,$G$4:$G$203,G136,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U136" s="92"/>
     </x:row>
     <x:row r="137" ht="22" customHeight="1">
       <x:c r="A137" s="70"/>
@@ -6525,6 +6964,7 @@
       <x:c r="T137" s="60" t="str">
         <x:f>IF(COUNTA(A137:D137)+COUNTA(G137:S137)=0,"",IF(OR(A137="",B137="",C137="",D137="",G137="",H137="",J137="",R137=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A137)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B137)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B137,$G$4:$G$203,G137,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U137" s="91"/>
     </x:row>
     <x:row r="138" ht="22" customHeight="1">
       <x:c r="A138" s="70"/>
@@ -6553,6 +6993,7 @@
       <x:c r="T138" s="60" t="str">
         <x:f>IF(COUNTA(A138:D138)+COUNTA(G138:S138)=0,"",IF(OR(A138="",B138="",C138="",D138="",G138="",H138="",J138="",R138=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A138)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B138)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B138,$G$4:$G$203,G138,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U138" s="92"/>
     </x:row>
     <x:row r="139" ht="22" customHeight="1">
       <x:c r="A139" s="70"/>
@@ -6581,6 +7022,7 @@
       <x:c r="T139" s="60" t="str">
         <x:f>IF(COUNTA(A139:D139)+COUNTA(G139:S139)=0,"",IF(OR(A139="",B139="",C139="",D139="",G139="",H139="",J139="",R139=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A139)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B139)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B139,$G$4:$G$203,G139,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U139" s="91"/>
     </x:row>
     <x:row r="140" ht="22" customHeight="1">
       <x:c r="A140" s="70"/>
@@ -6609,6 +7051,7 @@
       <x:c r="T140" s="60" t="str">
         <x:f>IF(COUNTA(A140:D140)+COUNTA(G140:S140)=0,"",IF(OR(A140="",B140="",C140="",D140="",G140="",H140="",J140="",R140=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A140)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B140)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B140,$G$4:$G$203,G140,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U140" s="92"/>
     </x:row>
     <x:row r="141" ht="22" customHeight="1">
       <x:c r="A141" s="70"/>
@@ -6637,6 +7080,7 @@
       <x:c r="T141" s="60" t="str">
         <x:f>IF(COUNTA(A141:D141)+COUNTA(G141:S141)=0,"",IF(OR(A141="",B141="",C141="",D141="",G141="",H141="",J141="",R141=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A141)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B141)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B141,$G$4:$G$203,G141,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U141" s="91"/>
     </x:row>
     <x:row r="142" ht="22" customHeight="1">
       <x:c r="A142" s="70"/>
@@ -6665,6 +7109,7 @@
       <x:c r="T142" s="60" t="str">
         <x:f>IF(COUNTA(A142:D142)+COUNTA(G142:S142)=0,"",IF(OR(A142="",B142="",C142="",D142="",G142="",H142="",J142="",R142=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A142)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B142)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B142,$G$4:$G$203,G142,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U142" s="92"/>
     </x:row>
     <x:row r="143" ht="22" customHeight="1">
       <x:c r="A143" s="70"/>
@@ -6693,6 +7138,7 @@
       <x:c r="T143" s="60" t="str">
         <x:f>IF(COUNTA(A143:D143)+COUNTA(G143:S143)=0,"",IF(OR(A143="",B143="",C143="",D143="",G143="",H143="",J143="",R143=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A143)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B143)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B143,$G$4:$G$203,G143,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U143" s="91"/>
     </x:row>
     <x:row r="144" ht="22" customHeight="1">
       <x:c r="A144" s="70"/>
@@ -6721,6 +7167,7 @@
       <x:c r="T144" s="60" t="str">
         <x:f>IF(COUNTA(A144:D144)+COUNTA(G144:S144)=0,"",IF(OR(A144="",B144="",C144="",D144="",G144="",H144="",J144="",R144=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A144)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B144)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B144,$G$4:$G$203,G144,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U144" s="92"/>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
       <x:c r="A145" s="70"/>
@@ -6749,6 +7196,7 @@
       <x:c r="T145" s="60" t="str">
         <x:f>IF(COUNTA(A145:D145)+COUNTA(G145:S145)=0,"",IF(OR(A145="",B145="",C145="",D145="",G145="",H145="",J145="",R145=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A145)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B145)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B145,$G$4:$G$203,G145,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U145" s="91"/>
     </x:row>
     <x:row r="146" ht="22" customHeight="1">
       <x:c r="A146" s="70"/>
@@ -6777,6 +7225,7 @@
       <x:c r="T146" s="60" t="str">
         <x:f>IF(COUNTA(A146:D146)+COUNTA(G146:S146)=0,"",IF(OR(A146="",B146="",C146="",D146="",G146="",H146="",J146="",R146=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A146)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B146)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B146,$G$4:$G$203,G146,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U146" s="92"/>
     </x:row>
     <x:row r="147" ht="22" customHeight="1">
       <x:c r="A147" s="70"/>
@@ -6805,6 +7254,7 @@
       <x:c r="T147" s="60" t="str">
         <x:f>IF(COUNTA(A147:D147)+COUNTA(G147:S147)=0,"",IF(OR(A147="",B147="",C147="",D147="",G147="",H147="",J147="",R147=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A147)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B147)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B147,$G$4:$G$203,G147,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U147" s="91"/>
     </x:row>
     <x:row r="148" ht="22" customHeight="1">
       <x:c r="A148" s="70"/>
@@ -6833,6 +7283,7 @@
       <x:c r="T148" s="60" t="str">
         <x:f>IF(COUNTA(A148:D148)+COUNTA(G148:S148)=0,"",IF(OR(A148="",B148="",C148="",D148="",G148="",H148="",J148="",R148=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A148)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B148)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B148,$G$4:$G$203,G148,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U148" s="92"/>
     </x:row>
     <x:row r="149" ht="22" customHeight="1">
       <x:c r="A149" s="70"/>
@@ -6861,6 +7312,7 @@
       <x:c r="T149" s="60" t="str">
         <x:f>IF(COUNTA(A149:D149)+COUNTA(G149:S149)=0,"",IF(OR(A149="",B149="",C149="",D149="",G149="",H149="",J149="",R149=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A149)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B149)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B149,$G$4:$G$203,G149,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U149" s="91"/>
     </x:row>
     <x:row r="150" ht="22" customHeight="1">
       <x:c r="A150" s="70"/>
@@ -6889,6 +7341,7 @@
       <x:c r="T150" s="60" t="str">
         <x:f>IF(COUNTA(A150:D150)+COUNTA(G150:S150)=0,"",IF(OR(A150="",B150="",C150="",D150="",G150="",H150="",J150="",R150=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A150)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B150)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B150,$G$4:$G$203,G150,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U150" s="92"/>
     </x:row>
     <x:row r="151" ht="22" customHeight="1">
       <x:c r="A151" s="70"/>
@@ -6917,6 +7370,7 @@
       <x:c r="T151" s="60" t="str">
         <x:f>IF(COUNTA(A151:D151)+COUNTA(G151:S151)=0,"",IF(OR(A151="",B151="",C151="",D151="",G151="",H151="",J151="",R151=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A151)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B151)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B151,$G$4:$G$203,G151,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U151" s="91"/>
     </x:row>
     <x:row r="152" ht="22" customHeight="1">
       <x:c r="A152" s="70"/>
@@ -6945,6 +7399,7 @@
       <x:c r="T152" s="60" t="str">
         <x:f>IF(COUNTA(A152:D152)+COUNTA(G152:S152)=0,"",IF(OR(A152="",B152="",C152="",D152="",G152="",H152="",J152="",R152=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A152)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B152)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B152,$G$4:$G$203,G152,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U152" s="92"/>
     </x:row>
     <x:row r="153" ht="22" customHeight="1">
       <x:c r="A153" s="70"/>
@@ -6973,6 +7428,7 @@
       <x:c r="T153" s="60" t="str">
         <x:f>IF(COUNTA(A153:D153)+COUNTA(G153:S153)=0,"",IF(OR(A153="",B153="",C153="",D153="",G153="",H153="",J153="",R153=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A153)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B153)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B153,$G$4:$G$203,G153,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U153" s="91"/>
     </x:row>
     <x:row r="154" ht="22" customHeight="1">
       <x:c r="A154" s="70"/>
@@ -7001,6 +7457,7 @@
       <x:c r="T154" s="60" t="str">
         <x:f>IF(COUNTA(A154:D154)+COUNTA(G154:S154)=0,"",IF(OR(A154="",B154="",C154="",D154="",G154="",H154="",J154="",R154=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A154)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B154)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B154,$G$4:$G$203,G154,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U154" s="92"/>
     </x:row>
     <x:row r="155" ht="22" customHeight="1">
       <x:c r="A155" s="70"/>
@@ -7029,6 +7486,7 @@
       <x:c r="T155" s="60" t="str">
         <x:f>IF(COUNTA(A155:D155)+COUNTA(G155:S155)=0,"",IF(OR(A155="",B155="",C155="",D155="",G155="",H155="",J155="",R155=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A155)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B155)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B155,$G$4:$G$203,G155,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U155" s="91"/>
     </x:row>
     <x:row r="156" ht="22" customHeight="1">
       <x:c r="A156" s="70"/>
@@ -7057,6 +7515,7 @@
       <x:c r="T156" s="60" t="str">
         <x:f>IF(COUNTA(A156:D156)+COUNTA(G156:S156)=0,"",IF(OR(A156="",B156="",C156="",D156="",G156="",H156="",J156="",R156=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A156)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B156)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B156,$G$4:$G$203,G156,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U156" s="92"/>
     </x:row>
     <x:row r="157" ht="22" customHeight="1">
       <x:c r="A157" s="70"/>
@@ -7085,6 +7544,7 @@
       <x:c r="T157" s="60" t="str">
         <x:f>IF(COUNTA(A157:D157)+COUNTA(G157:S157)=0,"",IF(OR(A157="",B157="",C157="",D157="",G157="",H157="",J157="",R157=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A157)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B157)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B157,$G$4:$G$203,G157,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U157" s="91"/>
     </x:row>
     <x:row r="158" ht="22" customHeight="1">
       <x:c r="A158" s="70"/>
@@ -7113,6 +7573,7 @@
       <x:c r="T158" s="60" t="str">
         <x:f>IF(COUNTA(A158:D158)+COUNTA(G158:S158)=0,"",IF(OR(A158="",B158="",C158="",D158="",G158="",H158="",J158="",R158=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A158)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B158)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B158,$G$4:$G$203,G158,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U158" s="92"/>
     </x:row>
     <x:row r="159" ht="22" customHeight="1">
       <x:c r="A159" s="70"/>
@@ -7141,6 +7602,7 @@
       <x:c r="T159" s="60" t="str">
         <x:f>IF(COUNTA(A159:D159)+COUNTA(G159:S159)=0,"",IF(OR(A159="",B159="",C159="",D159="",G159="",H159="",J159="",R159=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A159)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B159)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B159,$G$4:$G$203,G159,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U159" s="91"/>
     </x:row>
     <x:row r="160" ht="22" customHeight="1">
       <x:c r="A160" s="70"/>
@@ -7169,6 +7631,7 @@
       <x:c r="T160" s="60" t="str">
         <x:f>IF(COUNTA(A160:D160)+COUNTA(G160:S160)=0,"",IF(OR(A160="",B160="",C160="",D160="",G160="",H160="",J160="",R160=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A160)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B160)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B160,$G$4:$G$203,G160,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U160" s="92"/>
     </x:row>
     <x:row r="161" ht="22" customHeight="1">
       <x:c r="A161" s="70"/>
@@ -7197,6 +7660,7 @@
       <x:c r="T161" s="60" t="str">
         <x:f>IF(COUNTA(A161:D161)+COUNTA(G161:S161)=0,"",IF(OR(A161="",B161="",C161="",D161="",G161="",H161="",J161="",R161=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A161)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B161)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B161,$G$4:$G$203,G161,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U161" s="91"/>
     </x:row>
     <x:row r="162" ht="22" customHeight="1">
       <x:c r="A162" s="70"/>
@@ -7225,6 +7689,7 @@
       <x:c r="T162" s="60" t="str">
         <x:f>IF(COUNTA(A162:D162)+COUNTA(G162:S162)=0,"",IF(OR(A162="",B162="",C162="",D162="",G162="",H162="",J162="",R162=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A162)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B162)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B162,$G$4:$G$203,G162,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U162" s="92"/>
     </x:row>
     <x:row r="163" ht="22" customHeight="1">
       <x:c r="A163" s="70"/>
@@ -7253,6 +7718,7 @@
       <x:c r="T163" s="60" t="str">
         <x:f>IF(COUNTA(A163:D163)+COUNTA(G163:S163)=0,"",IF(OR(A163="",B163="",C163="",D163="",G163="",H163="",J163="",R163=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A163)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B163)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B163,$G$4:$G$203,G163,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U163" s="91"/>
     </x:row>
     <x:row r="164" ht="22" customHeight="1">
       <x:c r="A164" s="70"/>
@@ -7281,6 +7747,7 @@
       <x:c r="T164" s="60" t="str">
         <x:f>IF(COUNTA(A164:D164)+COUNTA(G164:S164)=0,"",IF(OR(A164="",B164="",C164="",D164="",G164="",H164="",J164="",R164=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A164)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B164)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B164,$G$4:$G$203,G164,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U164" s="92"/>
     </x:row>
     <x:row r="165" ht="22" customHeight="1">
       <x:c r="A165" s="70"/>
@@ -7309,6 +7776,7 @@
       <x:c r="T165" s="60" t="str">
         <x:f>IF(COUNTA(A165:D165)+COUNTA(G165:S165)=0,"",IF(OR(A165="",B165="",C165="",D165="",G165="",H165="",J165="",R165=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A165)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B165)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B165,$G$4:$G$203,G165,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U165" s="91"/>
     </x:row>
     <x:row r="166" ht="22" customHeight="1">
       <x:c r="A166" s="70"/>
@@ -7337,6 +7805,7 @@
       <x:c r="T166" s="60" t="str">
         <x:f>IF(COUNTA(A166:D166)+COUNTA(G166:S166)=0,"",IF(OR(A166="",B166="",C166="",D166="",G166="",H166="",J166="",R166=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A166)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B166)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B166,$G$4:$G$203,G166,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U166" s="92"/>
     </x:row>
     <x:row r="167" ht="22" customHeight="1">
       <x:c r="A167" s="70"/>
@@ -7365,6 +7834,7 @@
       <x:c r="T167" s="60" t="str">
         <x:f>IF(COUNTA(A167:D167)+COUNTA(G167:S167)=0,"",IF(OR(A167="",B167="",C167="",D167="",G167="",H167="",J167="",R167=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A167)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B167)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B167,$G$4:$G$203,G167,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U167" s="91"/>
     </x:row>
     <x:row r="168" ht="22" customHeight="1">
       <x:c r="A168" s="70"/>
@@ -7393,6 +7863,7 @@
       <x:c r="T168" s="60" t="str">
         <x:f>IF(COUNTA(A168:D168)+COUNTA(G168:S168)=0,"",IF(OR(A168="",B168="",C168="",D168="",G168="",H168="",J168="",R168=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A168)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B168)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B168,$G$4:$G$203,G168,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U168" s="92"/>
     </x:row>
     <x:row r="169" ht="22" customHeight="1">
       <x:c r="A169" s="70"/>
@@ -7421,6 +7892,7 @@
       <x:c r="T169" s="60" t="str">
         <x:f>IF(COUNTA(A169:D169)+COUNTA(G169:S169)=0,"",IF(OR(A169="",B169="",C169="",D169="",G169="",H169="",J169="",R169=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A169)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B169)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B169,$G$4:$G$203,G169,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U169" s="91"/>
     </x:row>
     <x:row r="170" ht="22" customHeight="1">
       <x:c r="A170" s="70"/>
@@ -7449,6 +7921,7 @@
       <x:c r="T170" s="60" t="str">
         <x:f>IF(COUNTA(A170:D170)+COUNTA(G170:S170)=0,"",IF(OR(A170="",B170="",C170="",D170="",G170="",H170="",J170="",R170=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A170)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B170)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B170,$G$4:$G$203,G170,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U170" s="92"/>
     </x:row>
     <x:row r="171" ht="22" customHeight="1">
       <x:c r="A171" s="70"/>
@@ -7477,6 +7950,7 @@
       <x:c r="T171" s="60" t="str">
         <x:f>IF(COUNTA(A171:D171)+COUNTA(G171:S171)=0,"",IF(OR(A171="",B171="",C171="",D171="",G171="",H171="",J171="",R171=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A171)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B171)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B171,$G$4:$G$203,G171,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U171" s="91"/>
     </x:row>
     <x:row r="172" ht="22" customHeight="1">
       <x:c r="A172" s="70"/>
@@ -7505,6 +7979,7 @@
       <x:c r="T172" s="60" t="str">
         <x:f>IF(COUNTA(A172:D172)+COUNTA(G172:S172)=0,"",IF(OR(A172="",B172="",C172="",D172="",G172="",H172="",J172="",R172=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A172)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B172)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B172,$G$4:$G$203,G172,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U172" s="92"/>
     </x:row>
     <x:row r="173" ht="22" customHeight="1">
       <x:c r="A173" s="70"/>
@@ -7533,6 +8008,7 @@
       <x:c r="T173" s="60" t="str">
         <x:f>IF(COUNTA(A173:D173)+COUNTA(G173:S173)=0,"",IF(OR(A173="",B173="",C173="",D173="",G173="",H173="",J173="",R173=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A173)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B173)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B173,$G$4:$G$203,G173,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U173" s="91"/>
     </x:row>
     <x:row r="174" ht="22" customHeight="1">
       <x:c r="A174" s="70"/>
@@ -7561,6 +8037,7 @@
       <x:c r="T174" s="60" t="str">
         <x:f>IF(COUNTA(A174:D174)+COUNTA(G174:S174)=0,"",IF(OR(A174="",B174="",C174="",D174="",G174="",H174="",J174="",R174=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A174)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B174)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B174,$G$4:$G$203,G174,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U174" s="92"/>
     </x:row>
     <x:row r="175" ht="22" customHeight="1">
       <x:c r="A175" s="70"/>
@@ -7589,6 +8066,7 @@
       <x:c r="T175" s="60" t="str">
         <x:f>IF(COUNTA(A175:D175)+COUNTA(G175:S175)=0,"",IF(OR(A175="",B175="",C175="",D175="",G175="",H175="",J175="",R175=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A175)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B175)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B175,$G$4:$G$203,G175,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U175" s="91"/>
     </x:row>
     <x:row r="176" ht="22" customHeight="1">
       <x:c r="A176" s="70"/>
@@ -7617,6 +8095,7 @@
       <x:c r="T176" s="60" t="str">
         <x:f>IF(COUNTA(A176:D176)+COUNTA(G176:S176)=0,"",IF(OR(A176="",B176="",C176="",D176="",G176="",H176="",J176="",R176=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A176)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B176)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B176,$G$4:$G$203,G176,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U176" s="92"/>
     </x:row>
     <x:row r="177" ht="22" customHeight="1">
       <x:c r="A177" s="70"/>
@@ -7645,6 +8124,7 @@
       <x:c r="T177" s="60" t="str">
         <x:f>IF(COUNTA(A177:D177)+COUNTA(G177:S177)=0,"",IF(OR(A177="",B177="",C177="",D177="",G177="",H177="",J177="",R177=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A177)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B177)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B177,$G$4:$G$203,G177,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U177" s="91"/>
     </x:row>
     <x:row r="178" ht="22" customHeight="1">
       <x:c r="A178" s="70"/>
@@ -7673,6 +8153,7 @@
       <x:c r="T178" s="60" t="str">
         <x:f>IF(COUNTA(A178:D178)+COUNTA(G178:S178)=0,"",IF(OR(A178="",B178="",C178="",D178="",G178="",H178="",J178="",R178=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A178)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B178)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B178,$G$4:$G$203,G178,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U178" s="92"/>
     </x:row>
     <x:row r="179" ht="22" customHeight="1">
       <x:c r="A179" s="70"/>
@@ -7701,6 +8182,7 @@
       <x:c r="T179" s="60" t="str">
         <x:f>IF(COUNTA(A179:D179)+COUNTA(G179:S179)=0,"",IF(OR(A179="",B179="",C179="",D179="",G179="",H179="",J179="",R179=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A179)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B179)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B179,$G$4:$G$203,G179,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U179" s="91"/>
     </x:row>
     <x:row r="180" ht="22" customHeight="1">
       <x:c r="A180" s="70"/>
@@ -7729,6 +8211,7 @@
       <x:c r="T180" s="60" t="str">
         <x:f>IF(COUNTA(A180:D180)+COUNTA(G180:S180)=0,"",IF(OR(A180="",B180="",C180="",D180="",G180="",H180="",J180="",R180=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A180)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B180)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B180,$G$4:$G$203,G180,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U180" s="92"/>
     </x:row>
     <x:row r="181" ht="22" customHeight="1">
       <x:c r="A181" s="70"/>
@@ -7757,6 +8240,7 @@
       <x:c r="T181" s="60" t="str">
         <x:f>IF(COUNTA(A181:D181)+COUNTA(G181:S181)=0,"",IF(OR(A181="",B181="",C181="",D181="",G181="",H181="",J181="",R181=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A181)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B181)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B181,$G$4:$G$203,G181,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U181" s="91"/>
     </x:row>
     <x:row r="182" ht="22" customHeight="1">
       <x:c r="A182" s="70"/>
@@ -7785,6 +8269,7 @@
       <x:c r="T182" s="60" t="str">
         <x:f>IF(COUNTA(A182:D182)+COUNTA(G182:S182)=0,"",IF(OR(A182="",B182="",C182="",D182="",G182="",H182="",J182="",R182=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A182)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B182)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B182,$G$4:$G$203,G182,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U182" s="92"/>
     </x:row>
     <x:row r="183" ht="22" customHeight="1">
       <x:c r="A183" s="70"/>
@@ -7813,6 +8298,7 @@
       <x:c r="T183" s="60" t="str">
         <x:f>IF(COUNTA(A183:D183)+COUNTA(G183:S183)=0,"",IF(OR(A183="",B183="",C183="",D183="",G183="",H183="",J183="",R183=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A183)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B183)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B183,$G$4:$G$203,G183,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U183" s="91"/>
     </x:row>
     <x:row r="184" ht="22" customHeight="1">
       <x:c r="A184" s="70"/>
@@ -7841,6 +8327,7 @@
       <x:c r="T184" s="60" t="str">
         <x:f>IF(COUNTA(A184:D184)+COUNTA(G184:S184)=0,"",IF(OR(A184="",B184="",C184="",D184="",G184="",H184="",J184="",R184=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A184)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B184)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B184,$G$4:$G$203,G184,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U184" s="92"/>
     </x:row>
     <x:row r="185" ht="22" customHeight="1">
       <x:c r="A185" s="70"/>
@@ -7869,6 +8356,7 @@
       <x:c r="T185" s="60" t="str">
         <x:f>IF(COUNTA(A185:D185)+COUNTA(G185:S185)=0,"",IF(OR(A185="",B185="",C185="",D185="",G185="",H185="",J185="",R185=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A185)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B185)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B185,$G$4:$G$203,G185,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U185" s="91"/>
     </x:row>
     <x:row r="186" ht="22" customHeight="1">
       <x:c r="A186" s="70"/>
@@ -7897,6 +8385,7 @@
       <x:c r="T186" s="60" t="str">
         <x:f>IF(COUNTA(A186:D186)+COUNTA(G186:S186)=0,"",IF(OR(A186="",B186="",C186="",D186="",G186="",H186="",J186="",R186=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A186)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B186)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B186,$G$4:$G$203,G186,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U186" s="92"/>
     </x:row>
     <x:row r="187" ht="22" customHeight="1">
       <x:c r="A187" s="70"/>
@@ -7925,6 +8414,7 @@
       <x:c r="T187" s="60" t="str">
         <x:f>IF(COUNTA(A187:D187)+COUNTA(G187:S187)=0,"",IF(OR(A187="",B187="",C187="",D187="",G187="",H187="",J187="",R187=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A187)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B187)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B187,$G$4:$G$203,G187,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U187" s="91"/>
     </x:row>
     <x:row r="188" ht="22" customHeight="1">
       <x:c r="A188" s="70"/>
@@ -7953,6 +8443,7 @@
       <x:c r="T188" s="60" t="str">
         <x:f>IF(COUNTA(A188:D188)+COUNTA(G188:S188)=0,"",IF(OR(A188="",B188="",C188="",D188="",G188="",H188="",J188="",R188=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A188)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B188)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B188,$G$4:$G$203,G188,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U188" s="92"/>
     </x:row>
     <x:row r="189" ht="22" customHeight="1">
       <x:c r="A189" s="70"/>
@@ -7981,6 +8472,7 @@
       <x:c r="T189" s="60" t="str">
         <x:f>IF(COUNTA(A189:D189)+COUNTA(G189:S189)=0,"",IF(OR(A189="",B189="",C189="",D189="",G189="",H189="",J189="",R189=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A189)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B189)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B189,$G$4:$G$203,G189,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U189" s="91"/>
     </x:row>
     <x:row r="190" ht="22" customHeight="1">
       <x:c r="A190" s="70"/>
@@ -8009,6 +8501,7 @@
       <x:c r="T190" s="60" t="str">
         <x:f>IF(COUNTA(A190:D190)+COUNTA(G190:S190)=0,"",IF(OR(A190="",B190="",C190="",D190="",G190="",H190="",J190="",R190=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A190)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B190)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B190,$G$4:$G$203,G190,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U190" s="92"/>
     </x:row>
     <x:row r="191" ht="22" customHeight="1">
       <x:c r="A191" s="70"/>
@@ -8037,6 +8530,7 @@
       <x:c r="T191" s="60" t="str">
         <x:f>IF(COUNTA(A191:D191)+COUNTA(G191:S191)=0,"",IF(OR(A191="",B191="",C191="",D191="",G191="",H191="",J191="",R191=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A191)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B191)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B191,$G$4:$G$203,G191,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U191" s="91"/>
     </x:row>
     <x:row r="192" ht="22" customHeight="1">
       <x:c r="A192" s="70"/>
@@ -8065,6 +8559,7 @@
       <x:c r="T192" s="60" t="str">
         <x:f>IF(COUNTA(A192:D192)+COUNTA(G192:S192)=0,"",IF(OR(A192="",B192="",C192="",D192="",G192="",H192="",J192="",R192=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A192)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B192)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B192,$G$4:$G$203,G192,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U192" s="92"/>
     </x:row>
     <x:row r="193" ht="22" customHeight="1">
       <x:c r="A193" s="70"/>
@@ -8093,6 +8588,7 @@
       <x:c r="T193" s="60" t="str">
         <x:f>IF(COUNTA(A193:D193)+COUNTA(G193:S193)=0,"",IF(OR(A193="",B193="",C193="",D193="",G193="",H193="",J193="",R193=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A193)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B193)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B193,$G$4:$G$203,G193,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U193" s="91"/>
     </x:row>
     <x:row r="194" ht="22" customHeight="1">
       <x:c r="A194" s="70"/>
@@ -8121,6 +8617,7 @@
       <x:c r="T194" s="60" t="str">
         <x:f>IF(COUNTA(A194:D194)+COUNTA(G194:S194)=0,"",IF(OR(A194="",B194="",C194="",D194="",G194="",H194="",J194="",R194=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A194)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B194)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B194,$G$4:$G$203,G194,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U194" s="92"/>
     </x:row>
     <x:row r="195" ht="22" customHeight="1">
       <x:c r="A195" s="70"/>
@@ -8149,6 +8646,7 @@
       <x:c r="T195" s="60" t="str">
         <x:f>IF(COUNTA(A195:D195)+COUNTA(G195:S195)=0,"",IF(OR(A195="",B195="",C195="",D195="",G195="",H195="",J195="",R195=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A195)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B195)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B195,$G$4:$G$203,G195,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U195" s="91"/>
     </x:row>
     <x:row r="196" ht="22" customHeight="1">
       <x:c r="A196" s="70"/>
@@ -8177,6 +8675,7 @@
       <x:c r="T196" s="60" t="str">
         <x:f>IF(COUNTA(A196:D196)+COUNTA(G196:S196)=0,"",IF(OR(A196="",B196="",C196="",D196="",G196="",H196="",J196="",R196=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A196)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B196)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B196,$G$4:$G$203,G196,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U196" s="92"/>
     </x:row>
     <x:row r="197" ht="22" customHeight="1">
       <x:c r="A197" s="70"/>
@@ -8205,6 +8704,7 @@
       <x:c r="T197" s="60" t="str">
         <x:f>IF(COUNTA(A197:D197)+COUNTA(G197:S197)=0,"",IF(OR(A197="",B197="",C197="",D197="",G197="",H197="",J197="",R197=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A197)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B197)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B197,$G$4:$G$203,G197,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U197" s="91"/>
     </x:row>
     <x:row r="198" ht="22" customHeight="1">
       <x:c r="A198" s="70"/>
@@ -8233,6 +8733,7 @@
       <x:c r="T198" s="60" t="str">
         <x:f>IF(COUNTA(A198:D198)+COUNTA(G198:S198)=0,"",IF(OR(A198="",B198="",C198="",D198="",G198="",H198="",J198="",R198=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A198)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B198)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B198,$G$4:$G$203,G198,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U198" s="92"/>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
       <x:c r="A199" s="70"/>
@@ -8261,6 +8762,7 @@
       <x:c r="T199" s="60" t="str">
         <x:f>IF(COUNTA(A199:D199)+COUNTA(G199:S199)=0,"",IF(OR(A199="",B199="",C199="",D199="",G199="",H199="",J199="",R199=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A199)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B199)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B199,$G$4:$G$203,G199,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U199" s="91"/>
     </x:row>
     <x:row r="200" ht="22" customHeight="1">
       <x:c r="A200" s="70"/>
@@ -8289,6 +8791,7 @@
       <x:c r="T200" s="60" t="str">
         <x:f>IF(COUNTA(A200:D200)+COUNTA(G200:S200)=0,"",IF(OR(A200="",B200="",C200="",D200="",G200="",H200="",J200="",R200=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A200)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B200)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B200,$G$4:$G$203,G200,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U200" s="92"/>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
       <x:c r="A201" s="70"/>
@@ -8317,6 +8820,7 @@
       <x:c r="T201" s="60" t="str">
         <x:f>IF(COUNTA(A201:D201)+COUNTA(G201:S201)=0,"",IF(OR(A201="",B201="",C201="",D201="",G201="",H201="",J201="",R201=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A201)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B201)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B201,$G$4:$G$203,G201,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U201" s="91"/>
     </x:row>
     <x:row r="202" ht="22" customHeight="1">
       <x:c r="A202" s="70"/>
@@ -8345,6 +8849,7 @@
       <x:c r="T202" s="60" t="str">
         <x:f>IF(COUNTA(A202:D202)+COUNTA(G202:S202)=0,"",IF(OR(A202="",B202="",C202="",D202="",G202="",H202="",J202="",R202=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A202)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B202)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B202,$G$4:$G$203,G202,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U202" s="92"/>
     </x:row>
     <x:row r="203" ht="22" customHeight="1">
       <x:c r="A203" s="72"/>
@@ -8373,11 +8878,12 @@
       <x:c r="T203" s="61" t="str">
         <x:f>IF(COUNTA(A203:D203)+COUNTA(G203:S203)=0,"",IF(OR(A203="",B203="",C203="",D203="",G203="",H203="",J203="",R203=""),"缺少必填项",IF(COUNTIF($A$4:$A$203,A203)&gt;1,"全局队伍ID重复",IF(COUNTIF('学校信息'!$A$4:$A$53,B203)=0,"学校ID不存在",IF(COUNTIFS($B$4:$B$203,B203,$G$4:$G$203,G203,$R$4:$R$203,"启用")&gt;1,"同校Hydro UID重复","通过")))))</x:f>
       </x:c>
+      <x:c r="U203" s="91"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:T1"/>
-    <x:mergeCell ref="A2:T2"/>
+    <x:mergeCell ref="A1:U1"/>
+    <x:mergeCell ref="A2:U2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A4:A203">
     <x:cfRule type="expression" dxfId="4" priority="1">
@@ -8406,7 +8912,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a2d66ca6ecf4fc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R604b11d7f9c742f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19082,7 +19588,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb832b1738ec14766"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree288c4fe0214800"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19448,6 +19954,90 @@
         <x:v>用于题目包和Checker一致性检查</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" s="109" t="str">
+        <x:v>校徽URL</x:v>
+      </x:c>
+      <x:c r="B15" s="108" t="str">
+        <x:v>完整 HTTP(S) URL 或安全根相对路径</x:v>
+      </x:c>
+      <x:c r="C15" s="108" t="str">
+        <x:v>/hydro-league-xcpcio/school-badges/school-a.png</x:v>
+      </x:c>
+      <x:c r="D15" s="108" t="str">
+        <x:v>根相对路径随 Hub 与学校 Agent 同源发布，适合浏览器无法访问公网的机房；禁止 //、反斜杠和 ..</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="109" t="str">
+        <x:v>奖牌分组</x:v>
+      </x:c>
+      <x:c r="B16" s="108" t="str">
+        <x:v>中文或英文；多项用逗号分隔</x:v>
+      </x:c>
+      <x:c r="C16" s="108" t="str">
+        <x:v>2025DKYCPC新生</x:v>
+      </x:c>
+      <x:c r="D16" s="108" t="str">
+        <x:v>不要填写保留组 official 或 unofficial</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="A17" s="109" t="str">
+        <x:v>奖牌设置</x:v>
+      </x:c>
+      <x:c r="B17" s="108" t="str">
+        <x:v>分组 + 3 个非负整数</x:v>
+      </x:c>
+      <x:c r="C17" s="108" t="str">
+        <x:v>2025DKYCPC新生 / 6 / 12 / 18</x:v>
+      </x:c>
+      <x:c r="D17" s="108" t="str">
+        <x:v>只控制 XCPCIO 显示，不推导人工奖项</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" s="109" t="str">
+        <x:v>奖项ID</x:v>
+      </x:c>
+      <x:c r="B18" s="108" t="str">
+        <x:v>字母或数字开头的稳定 ID</x:v>
+      </x:c>
+      <x:c r="C18" s="108" t="str">
+        <x:v>gold-medal</x:v>
+      </x:c>
+      <x:c r="D18" s="108" t="str">
+        <x:v>原样进入 Contest API/CDP；同一联赛内必须唯一</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="109" t="str">
+        <x:v>全局队伍ID列表</x:v>
+      </x:c>
+      <x:c r="B19" s="108" t="str">
+        <x:v>半角或全角逗号分隔</x:v>
+      </x:c>
+      <x:c r="C19" s="108" t="str">
+        <x:v>team-001,team-002</x:v>
+      </x:c>
+      <x:c r="D19" s="108" t="str">
+        <x:v>只能引用“启用”队伍；可留空表示无获奖队伍</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" s="109" t="str">
+        <x:v>停用队伍</x:v>
+      </x:c>
+      <x:c r="B20" s="108" t="str">
+        <x:v>启用状态填写“停用”</x:v>
+      </x:c>
+      <x:c r="C20" s="108" t="str">
+        <x:v>停用</x:v>
+      </x:c>
+      <x:c r="D20" s="108" t="str">
+        <x:v>不会进入中心配置，也不能被人工奖项引用</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -19455,4 +20045,902 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="95" t="str">
+        <x:v>XCPCIO 分组奖牌显示设置</x:v>
+      </x:c>
+      <x:c r="B1" s="95"/>
+      <x:c r="C1" s="95"/>
+      <x:c r="D1" s="95"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="99" t="str">
+        <x:v>可选表。分组必须被至少一支启用队伍使用；金、银、铜数量均填非负整数。此表只控制榜单奖牌分组与数量，不替代人工奖项。</x:v>
+      </x:c>
+      <x:c r="B2" s="99"/>
+      <x:c r="C2" s="99"/>
+      <x:c r="D2" s="99"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="87" t="str">
+        <x:v>分组</x:v>
+      </x:c>
+      <x:c r="B3" s="87" t="str">
+        <x:v>金牌数</x:v>
+      </x:c>
+      <x:c r="C3" s="87" t="str">
+        <x:v>银牌数</x:v>
+      </x:c>
+      <x:c r="D3" s="87" t="str">
+        <x:v>铜牌数</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="92"/>
+      <x:c r="B4" s="92"/>
+      <x:c r="C4" s="92"/>
+      <x:c r="D4" s="92"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="102"/>
+      <x:c r="B5" s="102"/>
+      <x:c r="C5" s="102"/>
+      <x:c r="D5" s="102"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="92"/>
+      <x:c r="B6" s="92"/>
+      <x:c r="C6" s="92"/>
+      <x:c r="D6" s="92"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="102"/>
+      <x:c r="B7" s="102"/>
+      <x:c r="C7" s="102"/>
+      <x:c r="D7" s="102"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="92"/>
+      <x:c r="B8" s="92"/>
+      <x:c r="C8" s="92"/>
+      <x:c r="D8" s="92"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="102"/>
+      <x:c r="B9" s="102"/>
+      <x:c r="C9" s="102"/>
+      <x:c r="D9" s="102"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="92"/>
+      <x:c r="B10" s="92"/>
+      <x:c r="C10" s="92"/>
+      <x:c r="D10" s="92"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="102"/>
+      <x:c r="B11" s="102"/>
+      <x:c r="C11" s="102"/>
+      <x:c r="D11" s="102"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="92"/>
+      <x:c r="B12" s="92"/>
+      <x:c r="C12" s="92"/>
+      <x:c r="D12" s="92"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="102"/>
+      <x:c r="B13" s="102"/>
+      <x:c r="C13" s="102"/>
+      <x:c r="D13" s="102"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="92"/>
+      <x:c r="B14" s="92"/>
+      <x:c r="C14" s="92"/>
+      <x:c r="D14" s="92"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="102"/>
+      <x:c r="B15" s="102"/>
+      <x:c r="C15" s="102"/>
+      <x:c r="D15" s="102"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="92"/>
+      <x:c r="B16" s="92"/>
+      <x:c r="C16" s="92"/>
+      <x:c r="D16" s="92"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="102"/>
+      <x:c r="B17" s="102"/>
+      <x:c r="C17" s="102"/>
+      <x:c r="D17" s="102"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="92"/>
+      <x:c r="B18" s="92"/>
+      <x:c r="C18" s="92"/>
+      <x:c r="D18" s="92"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="102"/>
+      <x:c r="B19" s="102"/>
+      <x:c r="C19" s="102"/>
+      <x:c r="D19" s="102"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="92"/>
+      <x:c r="B20" s="92"/>
+      <x:c r="C20" s="92"/>
+      <x:c r="D20" s="92"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="102"/>
+      <x:c r="B21" s="102"/>
+      <x:c r="C21" s="102"/>
+      <x:c r="D21" s="102"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="92"/>
+      <x:c r="B22" s="92"/>
+      <x:c r="C22" s="92"/>
+      <x:c r="D22" s="92"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="102"/>
+      <x:c r="B23" s="102"/>
+      <x:c r="C23" s="102"/>
+      <x:c r="D23" s="102"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="92"/>
+      <x:c r="B24" s="92"/>
+      <x:c r="C24" s="92"/>
+      <x:c r="D24" s="92"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="102"/>
+      <x:c r="B25" s="102"/>
+      <x:c r="C25" s="102"/>
+      <x:c r="D25" s="102"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="92"/>
+      <x:c r="B26" s="92"/>
+      <x:c r="C26" s="92"/>
+      <x:c r="D26" s="92"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="102"/>
+      <x:c r="B27" s="102"/>
+      <x:c r="C27" s="102"/>
+      <x:c r="D27" s="102"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="92"/>
+      <x:c r="B28" s="92"/>
+      <x:c r="C28" s="92"/>
+      <x:c r="D28" s="92"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="102"/>
+      <x:c r="B29" s="102"/>
+      <x:c r="C29" s="102"/>
+      <x:c r="D29" s="102"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="92"/>
+      <x:c r="B30" s="92"/>
+      <x:c r="C30" s="92"/>
+      <x:c r="D30" s="92"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="102"/>
+      <x:c r="B31" s="102"/>
+      <x:c r="C31" s="102"/>
+      <x:c r="D31" s="102"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="92"/>
+      <x:c r="B32" s="92"/>
+      <x:c r="C32" s="92"/>
+      <x:c r="D32" s="92"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="102"/>
+      <x:c r="B33" s="102"/>
+      <x:c r="C33" s="102"/>
+      <x:c r="D33" s="102"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="92"/>
+      <x:c r="B34" s="92"/>
+      <x:c r="C34" s="92"/>
+      <x:c r="D34" s="92"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="102"/>
+      <x:c r="B35" s="102"/>
+      <x:c r="C35" s="102"/>
+      <x:c r="D35" s="102"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="92"/>
+      <x:c r="B36" s="92"/>
+      <x:c r="C36" s="92"/>
+      <x:c r="D36" s="92"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="102"/>
+      <x:c r="B37" s="102"/>
+      <x:c r="C37" s="102"/>
+      <x:c r="D37" s="102"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="92"/>
+      <x:c r="B38" s="92"/>
+      <x:c r="C38" s="92"/>
+      <x:c r="D38" s="92"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="102"/>
+      <x:c r="B39" s="102"/>
+      <x:c r="C39" s="102"/>
+      <x:c r="D39" s="102"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="92"/>
+      <x:c r="B40" s="92"/>
+      <x:c r="C40" s="92"/>
+      <x:c r="D40" s="92"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="102"/>
+      <x:c r="B41" s="102"/>
+      <x:c r="C41" s="102"/>
+      <x:c r="D41" s="102"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="92"/>
+      <x:c r="B42" s="92"/>
+      <x:c r="C42" s="92"/>
+      <x:c r="D42" s="92"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="102"/>
+      <x:c r="B43" s="102"/>
+      <x:c r="C43" s="102"/>
+      <x:c r="D43" s="102"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="92"/>
+      <x:c r="B44" s="92"/>
+      <x:c r="C44" s="92"/>
+      <x:c r="D44" s="92"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="102"/>
+      <x:c r="B45" s="102"/>
+      <x:c r="C45" s="102"/>
+      <x:c r="D45" s="102"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="92"/>
+      <x:c r="B46" s="92"/>
+      <x:c r="C46" s="92"/>
+      <x:c r="D46" s="92"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="102"/>
+      <x:c r="B47" s="102"/>
+      <x:c r="C47" s="102"/>
+      <x:c r="D47" s="102"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="92"/>
+      <x:c r="B48" s="92"/>
+      <x:c r="C48" s="92"/>
+      <x:c r="D48" s="92"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="102"/>
+      <x:c r="B49" s="102"/>
+      <x:c r="C49" s="102"/>
+      <x:c r="D49" s="102"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="92"/>
+      <x:c r="B50" s="92"/>
+      <x:c r="C50" s="92"/>
+      <x:c r="D50" s="92"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="102"/>
+      <x:c r="B51" s="102"/>
+      <x:c r="C51" s="102"/>
+      <x:c r="D51" s="102"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="92"/>
+      <x:c r="B52" s="92"/>
+      <x:c r="C52" s="92"/>
+      <x:c r="D52" s="92"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="102"/>
+      <x:c r="B53" s="102"/>
+      <x:c r="C53" s="102"/>
+      <x:c r="D53" s="102"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="whole" operator="between" sqref="B4:D53">
+      <x:formula1>0</x:formula1>
+      <x:formula2>10000</x:formula2>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="38" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="95" t="str">
+        <x:v>ICPC Tools Resolver 人工奖项</x:v>
+      </x:c>
+      <x:c r="B1" s="95"/>
+      <x:c r="C1" s="95"/>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="99" t="str">
+        <x:v>可选表。奖项 ID 必须唯一；队伍 ID 以半角或全角逗号分隔，只能引用启用队伍。这里填写的名单是 CDP 与 Resolver 的权威奖项数据。</x:v>
+      </x:c>
+      <x:c r="B2" s="99"/>
+      <x:c r="C2" s="99"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="87" t="str">
+        <x:v>奖项ID</x:v>
+      </x:c>
+      <x:c r="B3" s="87" t="str">
+        <x:v>奖项名称</x:v>
+      </x:c>
+      <x:c r="C3" s="87" t="str">
+        <x:v>全局队伍ID列表</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="92"/>
+      <x:c r="B4" s="92"/>
+      <x:c r="C4" s="92"/>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="102"/>
+      <x:c r="B5" s="102"/>
+      <x:c r="C5" s="102"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="92"/>
+      <x:c r="B6" s="92"/>
+      <x:c r="C6" s="92"/>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="102"/>
+      <x:c r="B7" s="102"/>
+      <x:c r="C7" s="102"/>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="92"/>
+      <x:c r="B8" s="92"/>
+      <x:c r="C8" s="92"/>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="102"/>
+      <x:c r="B9" s="102"/>
+      <x:c r="C9" s="102"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="92"/>
+      <x:c r="B10" s="92"/>
+      <x:c r="C10" s="92"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="102"/>
+      <x:c r="B11" s="102"/>
+      <x:c r="C11" s="102"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="92"/>
+      <x:c r="B12" s="92"/>
+      <x:c r="C12" s="92"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="102"/>
+      <x:c r="B13" s="102"/>
+      <x:c r="C13" s="102"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="92"/>
+      <x:c r="B14" s="92"/>
+      <x:c r="C14" s="92"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="102"/>
+      <x:c r="B15" s="102"/>
+      <x:c r="C15" s="102"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="92"/>
+      <x:c r="B16" s="92"/>
+      <x:c r="C16" s="92"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="102"/>
+      <x:c r="B17" s="102"/>
+      <x:c r="C17" s="102"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="92"/>
+      <x:c r="B18" s="92"/>
+      <x:c r="C18" s="92"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="102"/>
+      <x:c r="B19" s="102"/>
+      <x:c r="C19" s="102"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="92"/>
+      <x:c r="B20" s="92"/>
+      <x:c r="C20" s="92"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="102"/>
+      <x:c r="B21" s="102"/>
+      <x:c r="C21" s="102"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="92"/>
+      <x:c r="B22" s="92"/>
+      <x:c r="C22" s="92"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="102"/>
+      <x:c r="B23" s="102"/>
+      <x:c r="C23" s="102"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="92"/>
+      <x:c r="B24" s="92"/>
+      <x:c r="C24" s="92"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="102"/>
+      <x:c r="B25" s="102"/>
+      <x:c r="C25" s="102"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="92"/>
+      <x:c r="B26" s="92"/>
+      <x:c r="C26" s="92"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="102"/>
+      <x:c r="B27" s="102"/>
+      <x:c r="C27" s="102"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="92"/>
+      <x:c r="B28" s="92"/>
+      <x:c r="C28" s="92"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="102"/>
+      <x:c r="B29" s="102"/>
+      <x:c r="C29" s="102"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="92"/>
+      <x:c r="B30" s="92"/>
+      <x:c r="C30" s="92"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="102"/>
+      <x:c r="B31" s="102"/>
+      <x:c r="C31" s="102"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="92"/>
+      <x:c r="B32" s="92"/>
+      <x:c r="C32" s="92"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="102"/>
+      <x:c r="B33" s="102"/>
+      <x:c r="C33" s="102"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="92"/>
+      <x:c r="B34" s="92"/>
+      <x:c r="C34" s="92"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="102"/>
+      <x:c r="B35" s="102"/>
+      <x:c r="C35" s="102"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="92"/>
+      <x:c r="B36" s="92"/>
+      <x:c r="C36" s="92"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="102"/>
+      <x:c r="B37" s="102"/>
+      <x:c r="C37" s="102"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="92"/>
+      <x:c r="B38" s="92"/>
+      <x:c r="C38" s="92"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="102"/>
+      <x:c r="B39" s="102"/>
+      <x:c r="C39" s="102"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="92"/>
+      <x:c r="B40" s="92"/>
+      <x:c r="C40" s="92"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="102"/>
+      <x:c r="B41" s="102"/>
+      <x:c r="C41" s="102"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="92"/>
+      <x:c r="B42" s="92"/>
+      <x:c r="C42" s="92"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="102"/>
+      <x:c r="B43" s="102"/>
+      <x:c r="C43" s="102"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="92"/>
+      <x:c r="B44" s="92"/>
+      <x:c r="C44" s="92"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="102"/>
+      <x:c r="B45" s="102"/>
+      <x:c r="C45" s="102"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="92"/>
+      <x:c r="B46" s="92"/>
+      <x:c r="C46" s="92"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="102"/>
+      <x:c r="B47" s="102"/>
+      <x:c r="C47" s="102"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="92"/>
+      <x:c r="B48" s="92"/>
+      <x:c r="C48" s="92"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="102"/>
+      <x:c r="B49" s="102"/>
+      <x:c r="C49" s="102"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="92"/>
+      <x:c r="B50" s="92"/>
+      <x:c r="C50" s="92"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="102"/>
+      <x:c r="B51" s="102"/>
+      <x:c r="C51" s="102"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="92"/>
+      <x:c r="B52" s="92"/>
+      <x:c r="C52" s="92"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="102"/>
+      <x:c r="B53" s="102"/>
+      <x:c r="C53" s="102"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="92"/>
+      <x:c r="B54" s="92"/>
+      <x:c r="C54" s="92"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="102"/>
+      <x:c r="B55" s="102"/>
+      <x:c r="C55" s="102"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="92"/>
+      <x:c r="B56" s="92"/>
+      <x:c r="C56" s="92"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="102"/>
+      <x:c r="B57" s="102"/>
+      <x:c r="C57" s="102"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="92"/>
+      <x:c r="B58" s="92"/>
+      <x:c r="C58" s="92"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="102"/>
+      <x:c r="B59" s="102"/>
+      <x:c r="C59" s="102"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="92"/>
+      <x:c r="B60" s="92"/>
+      <x:c r="C60" s="92"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="102"/>
+      <x:c r="B61" s="102"/>
+      <x:c r="C61" s="102"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="92"/>
+      <x:c r="B62" s="92"/>
+      <x:c r="C62" s="92"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="102"/>
+      <x:c r="B63" s="102"/>
+      <x:c r="C63" s="102"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="92"/>
+      <x:c r="B64" s="92"/>
+      <x:c r="C64" s="92"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="102"/>
+      <x:c r="B65" s="102"/>
+      <x:c r="C65" s="102"/>
+    </x:row>
+    <x:row r="66" ht="22" customHeight="1">
+      <x:c r="A66" s="92"/>
+      <x:c r="B66" s="92"/>
+      <x:c r="C66" s="92"/>
+    </x:row>
+    <x:row r="67" ht="22" customHeight="1">
+      <x:c r="A67" s="102"/>
+      <x:c r="B67" s="102"/>
+      <x:c r="C67" s="102"/>
+    </x:row>
+    <x:row r="68" ht="22" customHeight="1">
+      <x:c r="A68" s="92"/>
+      <x:c r="B68" s="92"/>
+      <x:c r="C68" s="92"/>
+    </x:row>
+    <x:row r="69" ht="22" customHeight="1">
+      <x:c r="A69" s="102"/>
+      <x:c r="B69" s="102"/>
+      <x:c r="C69" s="102"/>
+    </x:row>
+    <x:row r="70" ht="22" customHeight="1">
+      <x:c r="A70" s="92"/>
+      <x:c r="B70" s="92"/>
+      <x:c r="C70" s="92"/>
+    </x:row>
+    <x:row r="71" ht="22" customHeight="1">
+      <x:c r="A71" s="102"/>
+      <x:c r="B71" s="102"/>
+      <x:c r="C71" s="102"/>
+    </x:row>
+    <x:row r="72" ht="22" customHeight="1">
+      <x:c r="A72" s="92"/>
+      <x:c r="B72" s="92"/>
+      <x:c r="C72" s="92"/>
+    </x:row>
+    <x:row r="73" ht="22" customHeight="1">
+      <x:c r="A73" s="102"/>
+      <x:c r="B73" s="102"/>
+      <x:c r="C73" s="102"/>
+    </x:row>
+    <x:row r="74" ht="22" customHeight="1">
+      <x:c r="A74" s="92"/>
+      <x:c r="B74" s="92"/>
+      <x:c r="C74" s="92"/>
+    </x:row>
+    <x:row r="75" ht="22" customHeight="1">
+      <x:c r="A75" s="102"/>
+      <x:c r="B75" s="102"/>
+      <x:c r="C75" s="102"/>
+    </x:row>
+    <x:row r="76" ht="22" customHeight="1">
+      <x:c r="A76" s="92"/>
+      <x:c r="B76" s="92"/>
+      <x:c r="C76" s="92"/>
+    </x:row>
+    <x:row r="77" ht="22" customHeight="1">
+      <x:c r="A77" s="102"/>
+      <x:c r="B77" s="102"/>
+      <x:c r="C77" s="102"/>
+    </x:row>
+    <x:row r="78" ht="22" customHeight="1">
+      <x:c r="A78" s="92"/>
+      <x:c r="B78" s="92"/>
+      <x:c r="C78" s="92"/>
+    </x:row>
+    <x:row r="79" ht="22" customHeight="1">
+      <x:c r="A79" s="102"/>
+      <x:c r="B79" s="102"/>
+      <x:c r="C79" s="102"/>
+    </x:row>
+    <x:row r="80" ht="22" customHeight="1">
+      <x:c r="A80" s="92"/>
+      <x:c r="B80" s="92"/>
+      <x:c r="C80" s="92"/>
+    </x:row>
+    <x:row r="81" ht="22" customHeight="1">
+      <x:c r="A81" s="102"/>
+      <x:c r="B81" s="102"/>
+      <x:c r="C81" s="102"/>
+    </x:row>
+    <x:row r="82" ht="22" customHeight="1">
+      <x:c r="A82" s="92"/>
+      <x:c r="B82" s="92"/>
+      <x:c r="C82" s="92"/>
+    </x:row>
+    <x:row r="83" ht="22" customHeight="1">
+      <x:c r="A83" s="102"/>
+      <x:c r="B83" s="102"/>
+      <x:c r="C83" s="102"/>
+    </x:row>
+    <x:row r="84" ht="22" customHeight="1">
+      <x:c r="A84" s="92"/>
+      <x:c r="B84" s="92"/>
+      <x:c r="C84" s="92"/>
+    </x:row>
+    <x:row r="85" ht="22" customHeight="1">
+      <x:c r="A85" s="102"/>
+      <x:c r="B85" s="102"/>
+      <x:c r="C85" s="102"/>
+    </x:row>
+    <x:row r="86" ht="22" customHeight="1">
+      <x:c r="A86" s="92"/>
+      <x:c r="B86" s="92"/>
+      <x:c r="C86" s="92"/>
+    </x:row>
+    <x:row r="87" ht="22" customHeight="1">
+      <x:c r="A87" s="102"/>
+      <x:c r="B87" s="102"/>
+      <x:c r="C87" s="102"/>
+    </x:row>
+    <x:row r="88" ht="22" customHeight="1">
+      <x:c r="A88" s="92"/>
+      <x:c r="B88" s="92"/>
+      <x:c r="C88" s="92"/>
+    </x:row>
+    <x:row r="89" ht="22" customHeight="1">
+      <x:c r="A89" s="102"/>
+      <x:c r="B89" s="102"/>
+      <x:c r="C89" s="102"/>
+    </x:row>
+    <x:row r="90" ht="22" customHeight="1">
+      <x:c r="A90" s="92"/>
+      <x:c r="B90" s="92"/>
+      <x:c r="C90" s="92"/>
+    </x:row>
+    <x:row r="91" ht="22" customHeight="1">
+      <x:c r="A91" s="102"/>
+      <x:c r="B91" s="102"/>
+      <x:c r="C91" s="102"/>
+    </x:row>
+    <x:row r="92" ht="22" customHeight="1">
+      <x:c r="A92" s="92"/>
+      <x:c r="B92" s="92"/>
+      <x:c r="C92" s="92"/>
+    </x:row>
+    <x:row r="93" ht="22" customHeight="1">
+      <x:c r="A93" s="102"/>
+      <x:c r="B93" s="102"/>
+      <x:c r="C93" s="102"/>
+    </x:row>
+    <x:row r="94" ht="22" customHeight="1">
+      <x:c r="A94" s="92"/>
+      <x:c r="B94" s="92"/>
+      <x:c r="C94" s="92"/>
+    </x:row>
+    <x:row r="95" ht="22" customHeight="1">
+      <x:c r="A95" s="102"/>
+      <x:c r="B95" s="102"/>
+      <x:c r="C95" s="102"/>
+    </x:row>
+    <x:row r="96" ht="22" customHeight="1">
+      <x:c r="A96" s="92"/>
+      <x:c r="B96" s="92"/>
+      <x:c r="C96" s="92"/>
+    </x:row>
+    <x:row r="97" ht="22" customHeight="1">
+      <x:c r="A97" s="102"/>
+      <x:c r="B97" s="102"/>
+      <x:c r="C97" s="102"/>
+    </x:row>
+    <x:row r="98" ht="22" customHeight="1">
+      <x:c r="A98" s="92"/>
+      <x:c r="B98" s="92"/>
+      <x:c r="C98" s="92"/>
+    </x:row>
+    <x:row r="99" ht="22" customHeight="1">
+      <x:c r="A99" s="102"/>
+      <x:c r="B99" s="102"/>
+      <x:c r="C99" s="102"/>
+    </x:row>
+    <x:row r="100" ht="22" customHeight="1">
+      <x:c r="A100" s="92"/>
+      <x:c r="B100" s="92"/>
+      <x:c r="C100" s="92"/>
+    </x:row>
+    <x:row r="101" ht="22" customHeight="1">
+      <x:c r="A101" s="102"/>
+      <x:c r="B101" s="102"/>
+      <x:c r="C101" s="102"/>
+    </x:row>
+    <x:row r="102" ht="22" customHeight="1">
+      <x:c r="A102" s="92"/>
+      <x:c r="B102" s="92"/>
+      <x:c r="C102" s="92"/>
+    </x:row>
+    <x:row r="103" ht="22" customHeight="1">
+      <x:c r="A103" s="102"/>
+      <x:c r="B103" s="102"/>
+      <x:c r="C103" s="102"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A2:C2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>